<commit_message>
Modificacions del control EmpresesProducte. Afinant disseny BD
</commit_message>
<xml_diff>
--- a/Docs/AccesCotitzacionsEodHd.xlsx
+++ b/Docs/AccesCotitzacionsEodHd.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PC-HP11\naoj61\InversionsV3\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B9EAE5-F820-4D21-B7B6-8C032993837C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3316CB35-E4B7-4349-B4DA-D7CEE6C89E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" activeTab="1" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
+    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="42">
   <si>
     <t>US6701002056</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t>Data Tancament</t>
+  </si>
+  <si>
+    <t>Diferències entre EodHD i Real</t>
   </si>
 </sst>
 </file>
@@ -159,7 +162,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.000\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,6 +173,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -190,7 +201,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -251,11 +262,85 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -263,7 +348,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -271,6 +355,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -283,14 +373,210 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="27">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -965,319 +1251,1109 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF80A40C-7CB8-46A0-99EA-6106618D84CF}">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="21" width="11.81640625" customWidth="1"/>
+    <col min="2" max="3" width="9.26953125" customWidth="1"/>
+    <col min="4" max="4" width="9.26953125" style="7" customWidth="1"/>
+    <col min="5" max="11" width="9.26953125" customWidth="1"/>
+    <col min="12" max="19" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="17"/>
+      <c r="D1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="11" t="s">
+      <c r="E1" s="17"/>
+      <c r="F1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="11" t="s">
+      <c r="G1" s="17"/>
+      <c r="H1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="11" t="s">
+      <c r="I1" s="17"/>
+      <c r="J1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="12"/>
-      <c r="L1" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="12"/>
-      <c r="N1" s="9" t="s">
+      <c r="K1" s="17"/>
+      <c r="L1" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="O1" s="10"/>
-      <c r="P1" s="11" t="s">
+      <c r="M1" s="15"/>
+      <c r="N1" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="9" t="s">
+      <c r="O1" s="17"/>
+      <c r="P1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="10"/>
-      <c r="T1" s="9" t="s">
+      <c r="Q1" s="15"/>
+      <c r="R1" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="U1" s="10"/>
-    </row>
-    <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="13"/>
-      <c r="B2" s="6" t="s">
+      <c r="S1" s="15"/>
+    </row>
+    <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="19"/>
+      <c r="B2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="7" t="s">
+      <c r="L2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="P2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="T2" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A3" s="5">
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A3" s="9">
         <v>46078</v>
       </c>
-      <c r="B3" s="8">
-        <v>32.200000000000003</v>
-      </c>
-      <c r="C3" s="8">
-        <v>32.352691818567102</v>
-      </c>
-      <c r="D3" s="8">
+      <c r="B3" s="7">
         <v>32.159999999999997</v>
       </c>
-      <c r="E3" s="8">
+      <c r="C3" s="7">
         <f>238.4/7.4703</f>
         <v>31.913042314231024</v>
       </c>
-      <c r="F3" s="8">
+      <c r="D3" s="7">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="E3" s="7">
+        <v>32.352691818567102</v>
+      </c>
+      <c r="F3" s="7">
         <v>2.7</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>2.71</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="7">
         <v>427.9</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="7">
         <v>423.49700000000001</v>
       </c>
-      <c r="J3" s="8">
-        <v>417.75</v>
-      </c>
-      <c r="K3" s="8">
+      <c r="J3" s="7">
+        <v>423.75</v>
+      </c>
+      <c r="K3" s="7">
         <v>423.3</v>
       </c>
-      <c r="L3" s="8">
-        <v>34.69</v>
-      </c>
-      <c r="M3" s="8">
-        <v>34.195</v>
-      </c>
-      <c r="N3" s="8">
+      <c r="L3" s="7">
         <v>110.77</v>
       </c>
-      <c r="O3" s="8">
+      <c r="M3" s="7">
         <v>110.77</v>
       </c>
-      <c r="P3" s="8">
+      <c r="N3" s="7">
         <v>475.46769999999998</v>
       </c>
-      <c r="Q3" s="8">
+      <c r="O3" s="7">
         <v>475.46769999999998</v>
       </c>
-      <c r="R3" s="8">
+      <c r="P3" s="7">
         <v>56.211799999999997</v>
       </c>
-      <c r="S3" s="8">
+      <c r="Q3" s="7">
         <v>56.159389571852401</v>
       </c>
-      <c r="T3" s="8">
+      <c r="R3" s="7">
         <v>93.21</v>
       </c>
-      <c r="U3" s="8">
+      <c r="S3" s="7">
         <v>93.21</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A4" s="10">
         <v>46079</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
+        <v>31.87</v>
+      </c>
+      <c r="C4" s="7">
+        <v>31.9359674483349</v>
+      </c>
+      <c r="D4" s="7">
         <v>31.8</v>
       </c>
-      <c r="C4" s="8">
+      <c r="E4" s="7">
         <v>31.8678526048284</v>
       </c>
-      <c r="D4" s="8">
-        <v>31.87</v>
-      </c>
-      <c r="E4" s="8">
-        <v>31.9359674483349</v>
-      </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <v>2.7</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>2.7064803049555199</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>433.75</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="7">
         <v>432.06200000000001</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="7">
         <v>423.94</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="7">
         <v>423.3</v>
       </c>
-      <c r="L4" s="8">
-        <v>34.090000000000003</v>
-      </c>
-      <c r="M4" s="8">
-        <v>34.195</v>
-      </c>
-      <c r="N4" s="8">
+      <c r="L4" s="7">
         <v>110.77</v>
       </c>
-      <c r="O4" s="8">
+      <c r="M4" s="7">
         <v>110.77</v>
       </c>
-      <c r="P4" s="8">
+      <c r="N4" s="7">
         <v>475.49650000000003</v>
       </c>
-      <c r="Q4" s="8">
+      <c r="O4" s="7">
         <v>475.49650000000003</v>
       </c>
-      <c r="R4" s="8">
+      <c r="P4" s="7">
         <v>56.018300000000004</v>
       </c>
-      <c r="S4" s="8">
+      <c r="Q4" s="7">
         <v>56.0609911054637</v>
       </c>
-      <c r="T4" s="8">
+      <c r="R4" s="7">
         <v>93.23</v>
       </c>
-      <c r="U4" s="8">
+      <c r="S4" s="7">
         <v>93.23</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A5" s="5"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A6" s="5"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="8"/>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="H8" s="8"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="H9" s="8"/>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A5" s="10">
+        <v>46080</v>
+      </c>
+      <c r="B5" s="7">
+        <v>31.57</v>
+      </c>
+      <c r="C5" s="7">
+        <v>31.84</v>
+      </c>
+      <c r="D5" s="7">
+        <v>31.6</v>
+      </c>
+      <c r="E5" s="7">
+        <v>31.69</v>
+      </c>
+      <c r="F5" s="7">
+        <v>2.66</v>
+      </c>
+      <c r="G5" s="7">
+        <v>2.67</v>
+      </c>
+      <c r="H5" s="7">
+        <v>435.15</v>
+      </c>
+      <c r="I5" s="7">
+        <v>436.85</v>
+      </c>
+      <c r="J5" s="7">
+        <v>426.75</v>
+      </c>
+      <c r="K5" s="7">
+        <v>426.45</v>
+      </c>
+      <c r="L5" s="7">
+        <v>110.78</v>
+      </c>
+      <c r="M5" s="7">
+        <v>110.78</v>
+      </c>
+      <c r="N5" s="7">
+        <v>475.55650000000003</v>
+      </c>
+      <c r="O5" s="7">
+        <v>475.56</v>
+      </c>
+      <c r="P5" s="7">
+        <v>56.154200000000003</v>
+      </c>
+      <c r="Q5" s="7">
+        <v>56.1</v>
+      </c>
+      <c r="R5" s="7">
+        <v>93.23</v>
+      </c>
+      <c r="S5" s="7">
+        <v>93.23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A6" s="10">
+        <v>46082</v>
+      </c>
+      <c r="B6" s="7">
+        <v>31.4</v>
+      </c>
+      <c r="C6" s="7">
+        <v>30.99</v>
+      </c>
+      <c r="D6" s="7">
+        <v>31.45</v>
+      </c>
+      <c r="E6" s="7">
+        <v>31.61</v>
+      </c>
+      <c r="F6" s="7">
+        <v>2.66</v>
+      </c>
+      <c r="G6" s="7">
+        <v>2.68</v>
+      </c>
+      <c r="H6" s="7">
+        <v>451</v>
+      </c>
+      <c r="I6" s="7">
+        <v>440.14</v>
+      </c>
+      <c r="J6" s="7">
+        <v>413.85</v>
+      </c>
+      <c r="K6" s="7">
+        <v>413.7</v>
+      </c>
+      <c r="L6" s="7">
+        <v>110.77</v>
+      </c>
+      <c r="M6" s="7">
+        <v>110.77</v>
+      </c>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A7" s="10">
+        <v>46085</v>
+      </c>
+      <c r="B7" s="7">
+        <v>32.94</v>
+      </c>
+      <c r="C7" s="7">
+        <v>32.86</v>
+      </c>
+      <c r="D7" s="7">
+        <v>33.049999999999997</v>
+      </c>
+      <c r="E7" s="7">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="F7" s="7">
+        <v>2.7</v>
+      </c>
+      <c r="G7" s="7">
+        <v>2.73</v>
+      </c>
+      <c r="H7" s="7">
+        <v>448.85</v>
+      </c>
+      <c r="I7" s="7">
+        <v>448.68</v>
+      </c>
+      <c r="J7" s="7">
+        <v>418.75</v>
+      </c>
+      <c r="K7" s="7">
+        <v>418.85</v>
+      </c>
+      <c r="L7" s="7">
+        <v>110.78</v>
+      </c>
+      <c r="M7" s="7">
+        <v>110.77</v>
+      </c>
+      <c r="N7" s="7">
+        <v>475.60910000000001</v>
+      </c>
+      <c r="O7" s="7">
+        <v>475.60910000000001</v>
+      </c>
+      <c r="P7" s="7">
+        <v>56.58</v>
+      </c>
+      <c r="Q7" s="7">
+        <v>56.828763579927497</v>
+      </c>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A8" s="10">
+        <v>46086</v>
+      </c>
+      <c r="B8" s="7">
+        <v>33.33</v>
+      </c>
+      <c r="C8" s="7">
+        <v>33.289000000000001</v>
+      </c>
+      <c r="D8" s="7">
+        <v>33.549999999999997</v>
+      </c>
+      <c r="E8" s="7">
+        <v>33.613999999999997</v>
+      </c>
+      <c r="F8" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="G8" s="7">
+        <v>2.6669999999999998</v>
+      </c>
+      <c r="H8" s="7">
+        <v>449.65</v>
+      </c>
+      <c r="I8" s="7">
+        <v>450.62400000000002</v>
+      </c>
+      <c r="J8" s="7">
+        <v>430.55</v>
+      </c>
+      <c r="K8" s="7">
+        <v>429.05</v>
+      </c>
+      <c r="L8" s="7">
+        <v>110.78</v>
+      </c>
+      <c r="M8" s="7">
+        <v>110.78</v>
+      </c>
+      <c r="N8" s="7">
+        <v>475.62650000000002</v>
+      </c>
+      <c r="O8" s="7">
+        <v>475.62700000000001</v>
+      </c>
+      <c r="P8" s="7">
+        <v>56.756799999999998</v>
+      </c>
+      <c r="Q8" s="7">
+        <v>56.707000000000001</v>
+      </c>
+      <c r="R8" s="7">
+        <v>93.24</v>
+      </c>
+      <c r="S8" s="7">
+        <v>93.21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A9" s="10"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+    </row>
+    <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="10"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+    </row>
+    <row r="11" spans="1:19" ht="24" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A11" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="13"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
+        <f>A3</f>
+        <v>46078</v>
+      </c>
+      <c r="B12" s="8">
+        <f>C12</f>
+        <v>0.24695768576897237</v>
+      </c>
+      <c r="C12" s="8">
+        <f>B3-C3</f>
+        <v>0.24695768576897237</v>
+      </c>
+      <c r="D12" s="8">
+        <f>E12</f>
+        <v>-0.15269181856709935</v>
+      </c>
+      <c r="E12" s="8">
+        <f>D3-E3</f>
+        <v>-0.15269181856709935</v>
+      </c>
+      <c r="F12" s="8">
+        <f>G12</f>
+        <v>-9.9999999999997868E-3</v>
+      </c>
+      <c r="G12" s="8">
+        <f>F3-G3</f>
+        <v>-9.9999999999997868E-3</v>
+      </c>
+      <c r="H12" s="8">
+        <f>I12</f>
+        <v>4.4029999999999632</v>
+      </c>
+      <c r="I12" s="8">
+        <f>H3-I3</f>
+        <v>4.4029999999999632</v>
+      </c>
+      <c r="J12" s="8">
+        <f>K12</f>
+        <v>0.44999999999998863</v>
+      </c>
+      <c r="K12" s="8">
+        <f>J3-K3</f>
+        <v>0.44999999999998863</v>
+      </c>
+      <c r="L12" s="8">
+        <f>M12</f>
+        <v>0</v>
+      </c>
+      <c r="M12" s="8">
+        <f>L3-M3</f>
+        <v>0</v>
+      </c>
+      <c r="N12" s="8">
+        <f>O12</f>
+        <v>0</v>
+      </c>
+      <c r="O12" s="8">
+        <f>N3-O3</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="8">
+        <f>Q12</f>
+        <v>5.2410428147595667E-2</v>
+      </c>
+      <c r="Q12" s="8">
+        <f>P3-Q3</f>
+        <v>5.2410428147595667E-2</v>
+      </c>
+      <c r="R12" s="8">
+        <f>S12</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="8">
+        <f>R3-S3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A13" s="10">
+        <f>A4</f>
+        <v>46079</v>
+      </c>
+      <c r="B13" s="7">
+        <f>B12+C13</f>
+        <v>0.18099023743407372</v>
+      </c>
+      <c r="C13" s="7">
+        <f>B4-C4</f>
+        <v>-6.5967448334898648E-2</v>
+      </c>
+      <c r="D13" s="7">
+        <f>D12+E13</f>
+        <v>-0.22054442339549851</v>
+      </c>
+      <c r="E13" s="7">
+        <f>D4-E4</f>
+        <v>-6.7852604828399166E-2</v>
+      </c>
+      <c r="F13" s="7">
+        <f>F12+G13</f>
+        <v>-1.6480304955519554E-2</v>
+      </c>
+      <c r="G13" s="7">
+        <f>F4-G4</f>
+        <v>-6.4803049555197667E-3</v>
+      </c>
+      <c r="H13" s="7">
+        <f>H12+I13</f>
+        <v>6.0909999999999513</v>
+      </c>
+      <c r="I13" s="7">
+        <f>H4-I4</f>
+        <v>1.6879999999999882</v>
+      </c>
+      <c r="J13" s="7">
+        <f>J12+K13</f>
+        <v>1.089999999999975</v>
+      </c>
+      <c r="K13" s="7">
+        <f>J4-K4</f>
+        <v>0.63999999999998636</v>
+      </c>
+      <c r="L13" s="7">
+        <f>L12+M13</f>
+        <v>0</v>
+      </c>
+      <c r="M13" s="7">
+        <f>L4-M4</f>
+        <v>0</v>
+      </c>
+      <c r="N13" s="7">
+        <f>N12+O13</f>
+        <v>0</v>
+      </c>
+      <c r="O13" s="7">
+        <f>N4-O4</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="7">
+        <f>P12+Q13</f>
+        <v>9.7193226838996338E-3</v>
+      </c>
+      <c r="Q13" s="7">
+        <f>P4-Q4</f>
+        <v>-4.2691105463696033E-2</v>
+      </c>
+      <c r="R13" s="7">
+        <f>R12+S13</f>
+        <v>0</v>
+      </c>
+      <c r="S13" s="7">
+        <f>R4-S4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A14" s="10">
+        <f>A5</f>
+        <v>46080</v>
+      </c>
+      <c r="B14" s="7">
+        <f>B13+C14</f>
+        <v>-8.9009762565925854E-2</v>
+      </c>
+      <c r="C14" s="7">
+        <f>B5-C5</f>
+        <v>-0.26999999999999957</v>
+      </c>
+      <c r="D14" s="7">
+        <f>D13+E14</f>
+        <v>-0.31054442339549837</v>
+      </c>
+      <c r="E14" s="7">
+        <f>D5-E5</f>
+        <v>-8.9999999999999858E-2</v>
+      </c>
+      <c r="F14" s="7">
+        <f>F13+G14</f>
+        <v>-2.648030495551934E-2</v>
+      </c>
+      <c r="G14" s="7">
+        <f>F5-G5</f>
+        <v>-9.9999999999997868E-3</v>
+      </c>
+      <c r="H14" s="7">
+        <f>H13+I14</f>
+        <v>4.3909999999999059</v>
+      </c>
+      <c r="I14" s="7">
+        <f>H5-I5</f>
+        <v>-1.7000000000000455</v>
+      </c>
+      <c r="J14" s="7">
+        <f>J13+K14</f>
+        <v>1.3899999999999864</v>
+      </c>
+      <c r="K14" s="7">
+        <f>J5-K5</f>
+        <v>0.30000000000001137</v>
+      </c>
+      <c r="L14" s="7">
+        <f>L13+M14</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="7">
+        <f>L5-M5</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="7">
+        <f>N13+O14</f>
+        <v>-3.4999999999740794E-3</v>
+      </c>
+      <c r="O14" s="7">
+        <f>N5-O5</f>
+        <v>-3.4999999999740794E-3</v>
+      </c>
+      <c r="P14" s="7">
+        <f>P13+Q14</f>
+        <v>6.3919322683901214E-2</v>
+      </c>
+      <c r="Q14" s="7">
+        <f>P5-Q5</f>
+        <v>5.420000000000158E-2</v>
+      </c>
+      <c r="R14" s="7">
+        <f>R13+S14</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="7">
+        <f>R5-S5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A15" s="10">
+        <f>A6</f>
+        <v>46082</v>
+      </c>
+      <c r="B15" s="7">
+        <f>B14+C15</f>
+        <v>0.32099023743407429</v>
+      </c>
+      <c r="C15" s="7">
+        <f>B6-C6</f>
+        <v>0.41000000000000014</v>
+      </c>
+      <c r="D15" s="7">
+        <f>D14+E15</f>
+        <v>-0.47054442339549851</v>
+      </c>
+      <c r="E15" s="7">
+        <f>D6-E6</f>
+        <v>-0.16000000000000014</v>
+      </c>
+      <c r="F15" s="7">
+        <f>F14+G15</f>
+        <v>-4.6480304955519358E-2</v>
+      </c>
+      <c r="G15" s="7">
+        <f>F6-G6</f>
+        <v>-2.0000000000000018E-2</v>
+      </c>
+      <c r="H15" s="7">
+        <f>H14+I15</f>
+        <v>15.25099999999992</v>
+      </c>
+      <c r="I15" s="7">
+        <f>H6-I6</f>
+        <v>10.860000000000014</v>
+      </c>
+      <c r="J15" s="7">
+        <f>J14+K15</f>
+        <v>1.5400000000000205</v>
+      </c>
+      <c r="K15" s="7">
+        <f>J6-K6</f>
+        <v>0.15000000000003411</v>
+      </c>
+      <c r="L15" s="7">
+        <f>L14+M15</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="7">
+        <f>L6-M6</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="7">
+        <f>N14+O15</f>
+        <v>-3.4999999999740794E-3</v>
+      </c>
+      <c r="O15" s="7">
+        <f>N6-O6</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="7">
+        <f>P14+Q15</f>
+        <v>6.3919322683901214E-2</v>
+      </c>
+      <c r="Q15" s="7">
+        <f>P6-Q6</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="7">
+        <f>R14+S15</f>
+        <v>0</v>
+      </c>
+      <c r="S15" s="7">
+        <f>R6-S6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A16" s="10">
+        <f>A7</f>
+        <v>46085</v>
+      </c>
+      <c r="B16" s="7">
+        <f>B15+C16</f>
+        <v>0.40099023743407258</v>
+      </c>
+      <c r="C16" s="7">
+        <f>B7-C7</f>
+        <v>7.9999999999998295E-2</v>
+      </c>
+      <c r="D16" s="7">
+        <f>D15+E16</f>
+        <v>-0.6205444233955042</v>
+      </c>
+      <c r="E16" s="7">
+        <f>D7-E7</f>
+        <v>-0.15000000000000568</v>
+      </c>
+      <c r="F16" s="7">
+        <f>F15+G16</f>
+        <v>-7.6480304955519163E-2</v>
+      </c>
+      <c r="G16" s="7">
+        <f>F7-G7</f>
+        <v>-2.9999999999999805E-2</v>
+      </c>
+      <c r="H16" s="7">
+        <f>H15+I16</f>
+        <v>15.420999999999935</v>
+      </c>
+      <c r="I16" s="7">
+        <f>H7-I7</f>
+        <v>0.17000000000001592</v>
+      </c>
+      <c r="J16" s="7">
+        <f>J15+K16</f>
+        <v>1.4399999999999977</v>
+      </c>
+      <c r="K16" s="7">
+        <f>J7-K7</f>
+        <v>-0.10000000000002274</v>
+      </c>
+      <c r="L16" s="7">
+        <f>L15+M16</f>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="M16" s="7">
+        <f>L7-M7</f>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="N16" s="7">
+        <f>N15+O16</f>
+        <v>-3.4999999999740794E-3</v>
+      </c>
+      <c r="O16" s="7">
+        <f>N7-O7</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="7">
+        <f>P15+Q16</f>
+        <v>-0.1848442572435971</v>
+      </c>
+      <c r="Q16" s="7">
+        <f>P7-Q7</f>
+        <v>-0.24876357992749831</v>
+      </c>
+      <c r="R16" s="7">
+        <f>R15+S16</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="7">
+        <f>R7-S7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A17" s="10">
+        <f>A8</f>
+        <v>46086</v>
+      </c>
+      <c r="B17" s="7">
+        <f>B16+C17</f>
+        <v>0.4419902374340694</v>
+      </c>
+      <c r="C17" s="7">
+        <f>B8-C8</f>
+        <v>4.0999999999996817E-2</v>
+      </c>
+      <c r="D17" s="7">
+        <f>D16+E17</f>
+        <v>-0.68454442339550425</v>
+      </c>
+      <c r="E17" s="7">
+        <f>D8-E8</f>
+        <v>-6.4000000000000057E-2</v>
+      </c>
+      <c r="F17" s="7">
+        <f>F16+G17</f>
+        <v>-0.24348030495551898</v>
+      </c>
+      <c r="G17" s="7">
+        <f>F8-G8</f>
+        <v>-0.16699999999999982</v>
+      </c>
+      <c r="H17" s="7">
+        <f>H16+I17</f>
+        <v>14.446999999999889</v>
+      </c>
+      <c r="I17" s="7">
+        <f>H8-I8</f>
+        <v>-0.97400000000004638</v>
+      </c>
+      <c r="J17" s="7">
+        <f>J16+K17</f>
+        <v>2.9399999999999977</v>
+      </c>
+      <c r="K17" s="7">
+        <f>J8-K8</f>
+        <v>1.5</v>
+      </c>
+      <c r="L17" s="7">
+        <f>L16+M17</f>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="M17" s="7">
+        <f>L8-M8</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="7">
+        <f>N16+O17</f>
+        <v>-3.999999999962256E-3</v>
+      </c>
+      <c r="O17" s="7">
+        <f>N8-O8</f>
+        <v>-4.9999999998817657E-4</v>
+      </c>
+      <c r="P17" s="7">
+        <f>P16+Q17</f>
+        <v>-0.13504425724359947</v>
+      </c>
+      <c r="Q17" s="7">
+        <f>P8-Q8</f>
+        <v>4.9799999999997624E-2</v>
+      </c>
+      <c r="R17" s="7">
+        <f>R16+S17</f>
+        <v>3.0000000000001137E-2</v>
+      </c>
+      <c r="S17" s="7">
+        <f>R8-S8</f>
+        <v>3.0000000000001137E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="J22" s="7"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="J23" s="7"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="J24" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
+    <mergeCell ref="L1:M1"/>
     <mergeCell ref="N1:O1"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="R1:S1"/>
-    <mergeCell ref="T1:U1"/>
     <mergeCell ref="A1:A2"/>
+    <mergeCell ref="D1:E1"/>
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
-    <mergeCell ref="L1:M1"/>
   </mergeCells>
+  <conditionalFormatting sqref="E12:E17">
+    <cfRule type="expression" dxfId="26" priority="28">
+      <formula>AND(E12&gt;-1, E12&lt; 1, E12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="29">
+      <formula>E12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="30">
+      <formula>E12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12:C17">
+    <cfRule type="expression" dxfId="23" priority="25">
+      <formula>AND(C12&gt;-1, C12&lt; 1, C12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="26">
+      <formula>C12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="27">
+      <formula>C12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12:G17">
+    <cfRule type="expression" dxfId="20" priority="22">
+      <formula>AND(G12&gt;-1, G12&lt; 1, G12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="23">
+      <formula>G12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="24">
+      <formula>G12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I12:I17">
+    <cfRule type="expression" dxfId="17" priority="19">
+      <formula>AND(I12&gt;-1, I12&lt; 1, I12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="20">
+      <formula>I12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="21">
+      <formula>I12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12:K17">
+    <cfRule type="expression" dxfId="14" priority="16">
+      <formula>AND(K12&gt;-1, K12&lt; 1, K12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="17">
+      <formula>K12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="18">
+      <formula>K12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M12:M17">
+    <cfRule type="expression" dxfId="11" priority="10">
+      <formula>AND(M12&gt;-1, M12&lt; 1, M12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="11">
+      <formula>M12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="12">
+      <formula>M12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O12:O17">
+    <cfRule type="expression" dxfId="8" priority="7">
+      <formula>AND(O12&gt;-1, O12&lt; 1, O12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="8">
+      <formula>O12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="9">
+      <formula>O12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q12:Q17">
+    <cfRule type="expression" dxfId="5" priority="4">
+      <formula>AND(Q12&gt;-1, Q12&lt; 1, Q12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>Q12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>Q12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S12:S17">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>AND(S12&gt;-1, S12&lt; 1, S12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>S12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>S12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="F12:K14 L12:R14 E12:E16 G15:Q16 F15:F16 R15:T16" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Vaig pulint la BD i EmpresesProductesTab
</commit_message>
<xml_diff>
--- a/Docs/AccesCotitzacionsEodHd.xlsx
+++ b/Docs/AccesCotitzacionsEodHd.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PC-HP11\naoj61\InversionsV3\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3316CB35-E4B7-4349-B4DA-D7CEE6C89E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0EC216-C94B-48A6-8CE2-6B82ED61AAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" activeTab="1" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Updates" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="80">
   <si>
     <t>US6701002056</t>
   </si>
@@ -152,17 +153,132 @@
   </si>
   <si>
     <t>Diferències entre EodHD i Real</t>
+  </si>
+  <si>
+    <t>CLAR</t>
+  </si>
+  <si>
+    <t>CLAR.US</t>
+  </si>
+  <si>
+    <t>M4I.MU</t>
+  </si>
+  <si>
+    <t>BRYN.XETRA</t>
+  </si>
+  <si>
+    <t>NVO</t>
+  </si>
+  <si>
+    <t>NVO.US</t>
+  </si>
+  <si>
+    <t>NOVO-B</t>
+  </si>
+  <si>
+    <t>NOVO-B.CO</t>
+  </si>
+  <si>
+    <t>TickerExchange</t>
+  </si>
+  <si>
+    <t>LU0122612764.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0231459107.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0048621477.EUFUND</t>
+  </si>
+  <si>
+    <t>DE0008490962.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0108459040.EUFUND</t>
+  </si>
+  <si>
+    <t>ES0147711032.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0294221253.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0055114457.EUFUND</t>
+  </si>
+  <si>
+    <t>FR0010135103.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0300739322.EUFUND</t>
+  </si>
+  <si>
+    <t>HJUI.F</t>
+  </si>
+  <si>
+    <t>ES0125240038.EUFUND</t>
+  </si>
+  <si>
+    <t>ES0178521037.EUFUND</t>
+  </si>
+  <si>
+    <t>LU1213836080.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0090865873.EUFUND</t>
+  </si>
+  <si>
+    <t>ES0155598032.EUFUND</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Productes</t>
+  </si>
+  <si>
+    <t>LU0122377152.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0230918368.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0515769262.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0049014870.EUFUND</t>
+  </si>
+  <si>
+    <t>FR0010149161.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0171306680.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0128499588.EUFUND</t>
+  </si>
+  <si>
+    <t>LU0034353002.EUFUND</t>
+  </si>
+  <si>
+    <t>LU1235294995.EUFUND</t>
+  </si>
+  <si>
+    <t>LU1965927921.EUFUND</t>
+  </si>
+  <si>
+    <t>Productes_ProdAccions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.000\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,6 +301,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -340,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -361,6 +484,15 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -379,9 +511,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1251,7 +1387,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF80A40C-7CB8-46A0-99EA-6106618D84CF}">
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
@@ -1262,55 +1398,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="16" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17"/>
-      <c r="F1" s="16" t="s">
+      <c r="E1" s="20"/>
+      <c r="F1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="17"/>
-      <c r="H1" s="16" t="s">
+      <c r="G1" s="20"/>
+      <c r="H1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="17"/>
-      <c r="J1" s="16" t="s">
+      <c r="I1" s="20"/>
+      <c r="J1" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="17"/>
-      <c r="L1" s="14" t="s">
+      <c r="K1" s="20"/>
+      <c r="L1" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="15"/>
-      <c r="N1" s="16" t="s">
+      <c r="M1" s="18"/>
+      <c r="N1" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="O1" s="17"/>
-      <c r="P1" s="14" t="s">
+      <c r="O1" s="20"/>
+      <c r="P1" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="Q1" s="15"/>
-      <c r="R1" s="14" t="s">
+      <c r="Q1" s="18"/>
+      <c r="R1" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="S1" s="15"/>
+      <c r="S1" s="18"/>
     </row>
     <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="19"/>
+      <c r="A2" s="22"/>
       <c r="B2" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="14" t="s">
         <v>24</v>
       </c>
       <c r="E2" s="6" t="s">
@@ -1563,7 +1699,7 @@
         <v>451</v>
       </c>
       <c r="I6" s="7">
-        <v>440.14</v>
+        <v>450.14</v>
       </c>
       <c r="J6" s="7">
         <v>413.85</v>
@@ -1699,24 +1835,51 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A9" s="10"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="7"/>
-      <c r="S9" s="7"/>
+      <c r="A9" s="10">
+        <v>46087</v>
+      </c>
+      <c r="B9" s="7">
+        <v>33.15</v>
+      </c>
+      <c r="C9" s="25">
+        <v>33.183</v>
+      </c>
+      <c r="D9" s="25">
+        <v>33.15</v>
+      </c>
+      <c r="E9" s="25">
+        <v>33.195999999999998</v>
+      </c>
+      <c r="F9" s="25">
+        <v>2.56</v>
+      </c>
+      <c r="G9" s="25">
+        <v>2.573</v>
+      </c>
+      <c r="H9" s="25">
+        <v>447.15</v>
+      </c>
+      <c r="I9" s="25">
+        <v>450.36799999999999</v>
+      </c>
+      <c r="J9" s="25">
+        <v>429.05</v>
+      </c>
+      <c r="K9" s="25">
+        <v>424.95</v>
+      </c>
+      <c r="M9" s="25">
+        <v>110.79</v>
+      </c>
+      <c r="O9" s="25">
+        <v>475.66300000000001</v>
+      </c>
+      <c r="Q9" s="25">
+        <v>56.41</v>
+      </c>
+      <c r="S9">
+        <v>93.24</v>
+      </c>
     </row>
     <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="10"/>
@@ -1763,7 +1926,7 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
-        <f>A3</f>
+        <f t="shared" ref="A12:A18" si="0">A3</f>
         <v>46078</v>
       </c>
       <c r="B12" s="8">
@@ -1771,7 +1934,7 @@
         <v>0.24695768576897237</v>
       </c>
       <c r="C12" s="8">
-        <f>B3-C3</f>
+        <f t="shared" ref="C12:C17" si="1">B3-C3</f>
         <v>0.24695768576897237</v>
       </c>
       <c r="D12" s="8">
@@ -1779,7 +1942,7 @@
         <v>-0.15269181856709935</v>
       </c>
       <c r="E12" s="8">
-        <f>D3-E3</f>
+        <f t="shared" ref="E12:E17" si="2">D3-E3</f>
         <v>-0.15269181856709935</v>
       </c>
       <c r="F12" s="8">
@@ -1787,7 +1950,7 @@
         <v>-9.9999999999997868E-3</v>
       </c>
       <c r="G12" s="8">
-        <f>F3-G3</f>
+        <f t="shared" ref="G12:G17" si="3">F3-G3</f>
         <v>-9.9999999999997868E-3</v>
       </c>
       <c r="H12" s="8">
@@ -1795,7 +1958,7 @@
         <v>4.4029999999999632</v>
       </c>
       <c r="I12" s="8">
-        <f>H3-I3</f>
+        <f t="shared" ref="I12:I17" si="4">H3-I3</f>
         <v>4.4029999999999632</v>
       </c>
       <c r="J12" s="8">
@@ -1803,7 +1966,7 @@
         <v>0.44999999999998863</v>
       </c>
       <c r="K12" s="8">
-        <f>J3-K3</f>
+        <f t="shared" ref="K12:K17" si="5">J3-K3</f>
         <v>0.44999999999998863</v>
       </c>
       <c r="L12" s="8">
@@ -1811,7 +1974,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="8">
-        <f>L3-M3</f>
+        <f t="shared" ref="M12:M17" si="6">L3-M3</f>
         <v>0</v>
       </c>
       <c r="N12" s="8">
@@ -1819,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="8">
-        <f>N3-O3</f>
+        <f t="shared" ref="O12:O17" si="7">N3-O3</f>
         <v>0</v>
       </c>
       <c r="P12" s="8">
@@ -1827,7 +1990,7 @@
         <v>5.2410428147595667E-2</v>
       </c>
       <c r="Q12" s="8">
-        <f>P3-Q3</f>
+        <f t="shared" ref="Q12:Q17" si="8">P3-Q3</f>
         <v>5.2410428147595667E-2</v>
       </c>
       <c r="R12" s="8">
@@ -1835,13 +1998,13 @@
         <v>0</v>
       </c>
       <c r="S12" s="8">
-        <f>R3-S3</f>
+        <f t="shared" ref="S12:S17" si="9">R3-S3</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
-        <f>A4</f>
+        <f t="shared" si="0"/>
         <v>46079</v>
       </c>
       <c r="B13" s="7">
@@ -1849,7 +2012,7 @@
         <v>0.18099023743407372</v>
       </c>
       <c r="C13" s="7">
-        <f>B4-C4</f>
+        <f t="shared" si="1"/>
         <v>-6.5967448334898648E-2</v>
       </c>
       <c r="D13" s="7">
@@ -1857,7 +2020,7 @@
         <v>-0.22054442339549851</v>
       </c>
       <c r="E13" s="7">
-        <f>D4-E4</f>
+        <f t="shared" si="2"/>
         <v>-6.7852604828399166E-2</v>
       </c>
       <c r="F13" s="7">
@@ -1865,7 +2028,7 @@
         <v>-1.6480304955519554E-2</v>
       </c>
       <c r="G13" s="7">
-        <f>F4-G4</f>
+        <f t="shared" si="3"/>
         <v>-6.4803049555197667E-3</v>
       </c>
       <c r="H13" s="7">
@@ -1873,7 +2036,7 @@
         <v>6.0909999999999513</v>
       </c>
       <c r="I13" s="7">
-        <f>H4-I4</f>
+        <f t="shared" si="4"/>
         <v>1.6879999999999882</v>
       </c>
       <c r="J13" s="7">
@@ -1881,7 +2044,7 @@
         <v>1.089999999999975</v>
       </c>
       <c r="K13" s="7">
-        <f>J4-K4</f>
+        <f t="shared" si="5"/>
         <v>0.63999999999998636</v>
       </c>
       <c r="L13" s="7">
@@ -1889,7 +2052,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="7">
-        <f>L4-M4</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N13" s="7">
@@ -1897,7 +2060,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="7">
-        <f>N4-O4</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="P13" s="7">
@@ -1905,7 +2068,7 @@
         <v>9.7193226838996338E-3</v>
       </c>
       <c r="Q13" s="7">
-        <f>P4-Q4</f>
+        <f t="shared" si="8"/>
         <v>-4.2691105463696033E-2</v>
       </c>
       <c r="R13" s="7">
@@ -1913,13 +2076,13 @@
         <v>0</v>
       </c>
       <c r="S13" s="7">
-        <f>R4-S4</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14" s="10">
-        <f>A5</f>
+        <f t="shared" si="0"/>
         <v>46080</v>
       </c>
       <c r="B14" s="7">
@@ -1927,7 +2090,7 @@
         <v>-8.9009762565925854E-2</v>
       </c>
       <c r="C14" s="7">
-        <f>B5-C5</f>
+        <f t="shared" si="1"/>
         <v>-0.26999999999999957</v>
       </c>
       <c r="D14" s="7">
@@ -1935,7 +2098,7 @@
         <v>-0.31054442339549837</v>
       </c>
       <c r="E14" s="7">
-        <f>D5-E5</f>
+        <f t="shared" si="2"/>
         <v>-8.9999999999999858E-2</v>
       </c>
       <c r="F14" s="7">
@@ -1943,7 +2106,7 @@
         <v>-2.648030495551934E-2</v>
       </c>
       <c r="G14" s="7">
-        <f>F5-G5</f>
+        <f t="shared" si="3"/>
         <v>-9.9999999999997868E-3</v>
       </c>
       <c r="H14" s="7">
@@ -1951,7 +2114,7 @@
         <v>4.3909999999999059</v>
       </c>
       <c r="I14" s="7">
-        <f>H5-I5</f>
+        <f t="shared" si="4"/>
         <v>-1.7000000000000455</v>
       </c>
       <c r="J14" s="7">
@@ -1959,7 +2122,7 @@
         <v>1.3899999999999864</v>
       </c>
       <c r="K14" s="7">
-        <f>J5-K5</f>
+        <f t="shared" si="5"/>
         <v>0.30000000000001137</v>
       </c>
       <c r="L14" s="7">
@@ -1967,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="7">
-        <f>L5-M5</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N14" s="7">
@@ -1975,7 +2138,7 @@
         <v>-3.4999999999740794E-3</v>
       </c>
       <c r="O14" s="7">
-        <f>N5-O5</f>
+        <f t="shared" si="7"/>
         <v>-3.4999999999740794E-3</v>
       </c>
       <c r="P14" s="7">
@@ -1983,7 +2146,7 @@
         <v>6.3919322683901214E-2</v>
       </c>
       <c r="Q14" s="7">
-        <f>P5-Q5</f>
+        <f t="shared" si="8"/>
         <v>5.420000000000158E-2</v>
       </c>
       <c r="R14" s="7">
@@ -1991,13 +2154,13 @@
         <v>0</v>
       </c>
       <c r="S14" s="7">
-        <f>R5-S5</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
-        <f>A6</f>
+        <f t="shared" si="0"/>
         <v>46082</v>
       </c>
       <c r="B15" s="7">
@@ -2005,7 +2168,7 @@
         <v>0.32099023743407429</v>
       </c>
       <c r="C15" s="7">
-        <f>B6-C6</f>
+        <f t="shared" si="1"/>
         <v>0.41000000000000014</v>
       </c>
       <c r="D15" s="7">
@@ -2013,7 +2176,7 @@
         <v>-0.47054442339549851</v>
       </c>
       <c r="E15" s="7">
-        <f>D6-E6</f>
+        <f t="shared" si="2"/>
         <v>-0.16000000000000014</v>
       </c>
       <c r="F15" s="7">
@@ -2021,23 +2184,23 @@
         <v>-4.6480304955519358E-2</v>
       </c>
       <c r="G15" s="7">
-        <f>F6-G6</f>
+        <f t="shared" si="3"/>
         <v>-2.0000000000000018E-2</v>
       </c>
       <c r="H15" s="7">
         <f>H14+I15</f>
-        <v>15.25099999999992</v>
+        <v>5.2509999999999195</v>
       </c>
       <c r="I15" s="7">
-        <f>H6-I6</f>
-        <v>10.860000000000014</v>
+        <f t="shared" si="4"/>
+        <v>0.86000000000001364</v>
       </c>
       <c r="J15" s="7">
         <f>J14+K15</f>
         <v>1.5400000000000205</v>
       </c>
       <c r="K15" s="7">
-        <f>J6-K6</f>
+        <f t="shared" si="5"/>
         <v>0.15000000000003411</v>
       </c>
       <c r="L15" s="7">
@@ -2045,7 +2208,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="7">
-        <f>L6-M6</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N15" s="7">
@@ -2053,7 +2216,7 @@
         <v>-3.4999999999740794E-3</v>
       </c>
       <c r="O15" s="7">
-        <f>N6-O6</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="P15" s="7">
@@ -2061,7 +2224,7 @@
         <v>6.3919322683901214E-2</v>
       </c>
       <c r="Q15" s="7">
-        <f>P6-Q6</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="R15" s="7">
@@ -2069,13 +2232,13 @@
         <v>0</v>
       </c>
       <c r="S15" s="7">
-        <f>R6-S6</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
-        <f>A7</f>
+        <f t="shared" si="0"/>
         <v>46085</v>
       </c>
       <c r="B16" s="7">
@@ -2083,7 +2246,7 @@
         <v>0.40099023743407258</v>
       </c>
       <c r="C16" s="7">
-        <f>B7-C7</f>
+        <f t="shared" si="1"/>
         <v>7.9999999999998295E-2</v>
       </c>
       <c r="D16" s="7">
@@ -2091,7 +2254,7 @@
         <v>-0.6205444233955042</v>
       </c>
       <c r="E16" s="7">
-        <f>D7-E7</f>
+        <f t="shared" si="2"/>
         <v>-0.15000000000000568</v>
       </c>
       <c r="F16" s="7">
@@ -2099,15 +2262,15 @@
         <v>-7.6480304955519163E-2</v>
       </c>
       <c r="G16" s="7">
-        <f>F7-G7</f>
+        <f t="shared" si="3"/>
         <v>-2.9999999999999805E-2</v>
       </c>
       <c r="H16" s="7">
         <f>H15+I16</f>
-        <v>15.420999999999935</v>
+        <v>5.4209999999999354</v>
       </c>
       <c r="I16" s="7">
-        <f>H7-I7</f>
+        <f t="shared" si="4"/>
         <v>0.17000000000001592</v>
       </c>
       <c r="J16" s="7">
@@ -2115,7 +2278,7 @@
         <v>1.4399999999999977</v>
       </c>
       <c r="K16" s="7">
-        <f>J7-K7</f>
+        <f t="shared" si="5"/>
         <v>-0.10000000000002274</v>
       </c>
       <c r="L16" s="7">
@@ -2123,7 +2286,7 @@
         <v>1.0000000000005116E-2</v>
       </c>
       <c r="M16" s="7">
-        <f>L7-M7</f>
+        <f t="shared" si="6"/>
         <v>1.0000000000005116E-2</v>
       </c>
       <c r="N16" s="7">
@@ -2131,7 +2294,7 @@
         <v>-3.4999999999740794E-3</v>
       </c>
       <c r="O16" s="7">
-        <f>N7-O7</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="P16" s="7">
@@ -2139,7 +2302,7 @@
         <v>-0.1848442572435971</v>
       </c>
       <c r="Q16" s="7">
-        <f>P7-Q7</f>
+        <f t="shared" si="8"/>
         <v>-0.24876357992749831</v>
       </c>
       <c r="R16" s="7">
@@ -2147,13 +2310,13 @@
         <v>0</v>
       </c>
       <c r="S16" s="7">
-        <f>R7-S7</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
-        <f>A8</f>
+        <f t="shared" si="0"/>
         <v>46086</v>
       </c>
       <c r="B17" s="7">
@@ -2161,7 +2324,7 @@
         <v>0.4419902374340694</v>
       </c>
       <c r="C17" s="7">
-        <f>B8-C8</f>
+        <f t="shared" si="1"/>
         <v>4.0999999999996817E-2</v>
       </c>
       <c r="D17" s="7">
@@ -2169,7 +2332,7 @@
         <v>-0.68454442339550425</v>
       </c>
       <c r="E17" s="7">
-        <f>D8-E8</f>
+        <f t="shared" si="2"/>
         <v>-6.4000000000000057E-2</v>
       </c>
       <c r="F17" s="7">
@@ -2177,15 +2340,15 @@
         <v>-0.24348030495551898</v>
       </c>
       <c r="G17" s="7">
-        <f>F8-G8</f>
+        <f t="shared" si="3"/>
         <v>-0.16699999999999982</v>
       </c>
       <c r="H17" s="7">
         <f>H16+I17</f>
-        <v>14.446999999999889</v>
+        <v>4.446999999999889</v>
       </c>
       <c r="I17" s="7">
-        <f>H8-I8</f>
+        <f t="shared" si="4"/>
         <v>-0.97400000000004638</v>
       </c>
       <c r="J17" s="7">
@@ -2193,7 +2356,7 @@
         <v>2.9399999999999977</v>
       </c>
       <c r="K17" s="7">
-        <f>J8-K8</f>
+        <f t="shared" si="5"/>
         <v>1.5</v>
       </c>
       <c r="L17" s="7">
@@ -2201,7 +2364,7 @@
         <v>1.0000000000005116E-2</v>
       </c>
       <c r="M17" s="7">
-        <f>L8-M8</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N17" s="7">
@@ -2209,7 +2372,7 @@
         <v>-3.999999999962256E-3</v>
       </c>
       <c r="O17" s="7">
-        <f>N8-O8</f>
+        <f t="shared" si="7"/>
         <v>-4.9999999998817657E-4</v>
       </c>
       <c r="P17" s="7">
@@ -2217,7 +2380,7 @@
         <v>-0.13504425724359947</v>
       </c>
       <c r="Q17" s="7">
-        <f>P8-Q8</f>
+        <f t="shared" si="8"/>
         <v>4.9799999999997624E-2</v>
       </c>
       <c r="R17" s="7">
@@ -2225,18 +2388,59 @@
         <v>3.0000000000001137E-2</v>
       </c>
       <c r="S17" s="7">
-        <f>R8-S8</f>
+        <f t="shared" si="9"/>
         <v>3.0000000000001137E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="J22" s="7"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="J23" s="7"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="J24" s="7"/>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A18" s="10">
+        <f t="shared" si="0"/>
+        <v>46087</v>
+      </c>
+      <c r="B18" s="7">
+        <f>B17+C18</f>
+        <v>0.40899023743406815</v>
+      </c>
+      <c r="C18" s="7">
+        <f t="shared" ref="C18" si="10">B9-C9</f>
+        <v>-3.3000000000001251E-2</v>
+      </c>
+      <c r="D18" s="7">
+        <f>D17+E18</f>
+        <v>-0.73054442339550363</v>
+      </c>
+      <c r="E18" s="7">
+        <f t="shared" ref="E18" si="11">D9-E9</f>
+        <v>-4.5999999999999375E-2</v>
+      </c>
+      <c r="F18" s="7">
+        <f>F17+G18</f>
+        <v>-0.25648030495551888</v>
+      </c>
+      <c r="G18" s="7">
+        <f t="shared" ref="G18" si="12">F9-G9</f>
+        <v>-1.2999999999999901E-2</v>
+      </c>
+      <c r="H18" s="7">
+        <f>H17+I18</f>
+        <v>1.2289999999998713</v>
+      </c>
+      <c r="I18" s="7">
+        <f t="shared" ref="I18" si="13">H9-I9</f>
+        <v>-3.2180000000000177</v>
+      </c>
+      <c r="J18" s="7">
+        <f>J17+K18</f>
+        <v>7.0400000000000205</v>
+      </c>
+      <c r="K18" s="7">
+        <f t="shared" ref="K18" si="14">J9-K9</f>
+        <v>4.1000000000000227</v>
+      </c>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2251,29 +2455,29 @@
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E12:E17">
-    <cfRule type="expression" dxfId="26" priority="28">
+  <conditionalFormatting sqref="C12:C18">
+    <cfRule type="expression" dxfId="26" priority="25">
+      <formula>AND(C12&gt;-1, C12&lt; 1, C12 &lt;&gt; 0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="26">
+      <formula>C12&lt;=-1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="27">
+      <formula>C12&gt;=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12:E18">
+    <cfRule type="expression" dxfId="23" priority="28">
       <formula>AND(E12&gt;-1, E12&lt; 1, E12 &lt;&gt; 0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="29">
+    <cfRule type="expression" dxfId="22" priority="29">
       <formula>E12&lt;=-1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="30">
+    <cfRule type="expression" dxfId="21" priority="30">
       <formula>E12&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C12:C17">
-    <cfRule type="expression" dxfId="23" priority="25">
-      <formula>AND(C12&gt;-1, C12&lt; 1, C12 &lt;&gt; 0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="26">
-      <formula>C12&lt;=-1</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="21" priority="27">
-      <formula>C12&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G12:G17">
+  <conditionalFormatting sqref="G12:G18">
     <cfRule type="expression" dxfId="20" priority="22">
       <formula>AND(G12&gt;-1, G12&lt; 1, G12 &lt;&gt; 0)</formula>
     </cfRule>
@@ -2284,7 +2488,7 @@
       <formula>G12&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I12:I17">
+  <conditionalFormatting sqref="I12:I18">
     <cfRule type="expression" dxfId="17" priority="19">
       <formula>AND(I12&gt;-1, I12&lt; 1, I12 &lt;&gt; 0)</formula>
     </cfRule>
@@ -2295,7 +2499,7 @@
       <formula>I12&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K12:K17">
+  <conditionalFormatting sqref="K12:K18">
     <cfRule type="expression" dxfId="14" priority="16">
       <formula>AND(K12&gt;-1, K12&lt; 1, K12 &lt;&gt; 0)</formula>
     </cfRule>
@@ -2306,7 +2510,7 @@
       <formula>K12&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M12:M17">
+  <conditionalFormatting sqref="M12:M18">
     <cfRule type="expression" dxfId="11" priority="10">
       <formula>AND(M12&gt;-1, M12&lt; 1, M12 &lt;&gt; 0)</formula>
     </cfRule>
@@ -2317,7 +2521,7 @@
       <formula>M12&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O12:O17">
+  <conditionalFormatting sqref="O12:O18">
     <cfRule type="expression" dxfId="8" priority="7">
       <formula>AND(O12&gt;-1, O12&lt; 1, O12 &lt;&gt; 0)</formula>
     </cfRule>
@@ -2356,4 +2560,493 @@
     <ignoredError sqref="F12:K14 L12:R14 E12:E16 G15:Q16 F15:F16 R15:T16" formula="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D45F4E0-DDC0-44AE-A48F-B33A7D849191}">
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="73.54296875" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.453125" customWidth="1"/>
+    <col min="5" max="5" width="9.54296875" customWidth="1"/>
+    <col min="6" max="6" width="13.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B1" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="23"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="B2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="str">
+        <f>"UPDATE Productes SET TickerExchange = '"&amp;C3&amp;"' WHERE Id = "&amp;B3&amp;";"</f>
+        <v>UPDATE Productes SET TickerExchange = 'LU0122612764.EUFUND' WHERE Id = 2;</v>
+      </c>
+      <c r="B3" s="16">
+        <v>2</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="str">
+        <f t="shared" ref="A4:A33" si="0">"UPDATE Productes SET TickerExchange = '"&amp;C4&amp;"' WHERE Id = "&amp;B4&amp;";"</f>
+        <v>UPDATE Productes SET TickerExchange = 'LU0231459107.EUFUND' WHERE Id = 3;</v>
+      </c>
+      <c r="B4" s="16">
+        <v>3</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0048621477.EUFUND' WHERE Id = 4;</v>
+      </c>
+      <c r="B5" s="16">
+        <v>4</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'DE0008490962.EUFUND' WHERE Id = 5;</v>
+      </c>
+      <c r="B6" s="16">
+        <v>5</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0108459040.EUFUND' WHERE Id = 6;</v>
+      </c>
+      <c r="B7" s="16">
+        <v>6</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'ES0147711032.EUFUND' WHERE Id = 10;</v>
+      </c>
+      <c r="B8" s="16">
+        <v>10</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0294221253.EUFUND' WHERE Id = 11;</v>
+      </c>
+      <c r="B9" s="16">
+        <v>11</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0055114457.EUFUND' WHERE Id = 13;</v>
+      </c>
+      <c r="B10" s="16">
+        <v>13</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'FR0010135103.EUFUND' WHERE Id = 14;</v>
+      </c>
+      <c r="B11" s="16">
+        <v>14</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0300739322.EUFUND' WHERE Id = 15;</v>
+      </c>
+      <c r="B12" s="16">
+        <v>15</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'HJUI.F' WHERE Id = 16;</v>
+      </c>
+      <c r="B13" s="16">
+        <v>16</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'ES0125240038.EUFUND' WHERE Id = 19;</v>
+      </c>
+      <c r="B14" s="16">
+        <v>19</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'ES0178521037.EUFUND' WHERE Id = 26;</v>
+      </c>
+      <c r="B15" s="16">
+        <v>26</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU1213836080.EUFUND' WHERE Id = 27;</v>
+      </c>
+      <c r="B16" s="16">
+        <v>27</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0090865873.EUFUND' WHERE Id = 28;</v>
+      </c>
+      <c r="B17" s="16">
+        <v>28</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'ES0155598032.EUFUND' WHERE Id = 29;</v>
+      </c>
+      <c r="B18" s="16">
+        <v>29</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0122377152.EUFUND' WHERE Id = 30;</v>
+      </c>
+      <c r="B19" s="16">
+        <v>30</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0230918368.EUFUND' WHERE Id = 1036;</v>
+      </c>
+      <c r="B20" s="16">
+        <v>1036</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0515769262.EUFUND' WHERE Id = 1037;</v>
+      </c>
+      <c r="B21" s="16">
+        <v>1037</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0049014870.EUFUND' WHERE Id = 1038;</v>
+      </c>
+      <c r="B22" s="16">
+        <v>1038</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'FR0010149161.EUFUND' WHERE Id = 1039;</v>
+      </c>
+      <c r="B23" s="16">
+        <v>1039</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0171306680.EUFUND' WHERE Id = 1040;</v>
+      </c>
+      <c r="B24" s="16">
+        <v>1040</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0128499588.EUFUND' WHERE Id = 1041;</v>
+      </c>
+      <c r="B25" s="16">
+        <v>1041</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU0034353002.EUFUND' WHERE Id = 1042;</v>
+      </c>
+      <c r="B26" s="16">
+        <v>1042</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU1235294995.EUFUND' WHERE Id = 1043;</v>
+      </c>
+      <c r="B27" s="16">
+        <v>1043</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'CLAR.US' WHERE Id = 1045;</v>
+      </c>
+      <c r="B28" s="16">
+        <v>1045</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU1965927921.EUFUND' WHERE Id = 1046;</v>
+      </c>
+      <c r="B29" s="16">
+        <v>1046</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'M4I.MU' WHERE Id = 1053;</v>
+      </c>
+      <c r="B30" s="16">
+        <v>1053</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'BRYN.XETRA' WHERE Id = 1054;</v>
+      </c>
+      <c r="B31" s="16">
+        <v>1054</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'NVO.US' WHERE Id = 1058;</v>
+      </c>
+      <c r="B32" s="16">
+        <v>1058</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'NOVO-B.CO' WHERE Id = 1059;</v>
+      </c>
+      <c r="B33" s="16">
+        <v>1059</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B35" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="23"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B36" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="str">
+        <f>"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C37&amp;"' WHERE Id = "&amp;B37&amp;";"</f>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'CLAR' WHERE Id = 1045;</v>
+      </c>
+      <c r="B37" s="15">
+        <v>1045</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="str">
+        <f t="shared" ref="A38:A41" si="1">"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C38&amp;"' WHERE Id = "&amp;B38&amp;";"</f>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'M4I' WHERE Id = 1053;</v>
+      </c>
+      <c r="B38" s="15">
+        <v>1053</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'BRYN' WHERE Id = 1054;</v>
+      </c>
+      <c r="B39" s="15">
+        <v>1054</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'NVO' WHERE Id = 1058;</v>
+      </c>
+      <c r="B40" s="15">
+        <v>1058</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'NOVO-B' WHERE Id = 1059;</v>
+      </c>
+      <c r="B41" s="15">
+        <v>1059</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B35:C35"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Això ja gairebé està.
</commit_message>
<xml_diff>
--- a/Docs/AccesCotitzacionsEodHd.xlsx
+++ b/Docs/AccesCotitzacionsEodHd.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PC-HP11\naoj61\InversionsV3\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0EC216-C94B-48A6-8CE2-6B82ED61AAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542899D6-0B67-4089-9FB9-3605101340DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" activeTab="1" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
+    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="91">
   <si>
     <t>US6701002056</t>
   </si>
@@ -267,6 +267,39 @@
   </si>
   <si>
     <t>Productes_ProdAccions</t>
+  </si>
+  <si>
+    <t>MTS.AU</t>
+  </si>
+  <si>
+    <t>SAN.MC</t>
+  </si>
+  <si>
+    <t>TEF.MC</t>
+  </si>
+  <si>
+    <t>SAB.VN</t>
+  </si>
+  <si>
+    <t>ITX.MC</t>
+  </si>
+  <si>
+    <t>MTS</t>
+  </si>
+  <si>
+    <t>SAN</t>
+  </si>
+  <si>
+    <t>TEF</t>
+  </si>
+  <si>
+    <t>SAB</t>
+  </si>
+  <si>
+    <t>ITX</t>
+  </si>
+  <si>
+    <t>NDUEEGF</t>
   </si>
 </sst>
 </file>
@@ -493,6 +526,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -514,10 +551,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1398,48 +1431,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="19" t="s">
+      <c r="C1" s="22"/>
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20"/>
-      <c r="F1" s="19" t="s">
+      <c r="E1" s="22"/>
+      <c r="F1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="19" t="s">
+      <c r="G1" s="22"/>
+      <c r="H1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="20"/>
-      <c r="J1" s="19" t="s">
+      <c r="I1" s="22"/>
+      <c r="J1" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="20"/>
-      <c r="L1" s="17" t="s">
+      <c r="K1" s="22"/>
+      <c r="L1" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="18"/>
-      <c r="N1" s="19" t="s">
+      <c r="M1" s="20"/>
+      <c r="N1" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="O1" s="20"/>
-      <c r="P1" s="17" t="s">
+      <c r="O1" s="22"/>
+      <c r="P1" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="17" t="s">
+      <c r="Q1" s="20"/>
+      <c r="R1" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="S1" s="18"/>
+      <c r="S1" s="20"/>
     </row>
     <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="22"/>
+      <c r="A2" s="24"/>
       <c r="B2" s="5" t="s">
         <v>24</v>
       </c>
@@ -1841,40 +1874,40 @@
       <c r="B9" s="7">
         <v>33.15</v>
       </c>
-      <c r="C9" s="25">
+      <c r="C9" s="18">
         <v>33.183</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="18">
         <v>33.15</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="18">
         <v>33.195999999999998</v>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="18">
         <v>2.56</v>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="18">
         <v>2.573</v>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="18">
         <v>447.15</v>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="18">
         <v>450.36799999999999</v>
       </c>
-      <c r="J9" s="25">
+      <c r="J9" s="18">
         <v>429.05</v>
       </c>
-      <c r="K9" s="25">
+      <c r="K9" s="18">
         <v>424.95</v>
       </c>
-      <c r="M9" s="25">
+      <c r="M9" s="18">
         <v>110.79</v>
       </c>
-      <c r="O9" s="25">
+      <c r="O9" s="18">
         <v>475.66300000000001</v>
       </c>
-      <c r="Q9" s="25">
+      <c r="Q9" s="18">
         <v>56.41</v>
       </c>
       <c r="S9">
@@ -2008,7 +2041,7 @@
         <v>46079</v>
       </c>
       <c r="B13" s="7">
-        <f>B12+C13</f>
+        <f t="shared" ref="B13:B18" si="10">B12+C13</f>
         <v>0.18099023743407372</v>
       </c>
       <c r="C13" s="7">
@@ -2016,7 +2049,7 @@
         <v>-6.5967448334898648E-2</v>
       </c>
       <c r="D13" s="7">
-        <f>D12+E13</f>
+        <f t="shared" ref="D13:D18" si="11">D12+E13</f>
         <v>-0.22054442339549851</v>
       </c>
       <c r="E13" s="7">
@@ -2024,7 +2057,7 @@
         <v>-6.7852604828399166E-2</v>
       </c>
       <c r="F13" s="7">
-        <f>F12+G13</f>
+        <f t="shared" ref="F13:F18" si="12">F12+G13</f>
         <v>-1.6480304955519554E-2</v>
       </c>
       <c r="G13" s="7">
@@ -2032,7 +2065,7 @@
         <v>-6.4803049555197667E-3</v>
       </c>
       <c r="H13" s="7">
-        <f>H12+I13</f>
+        <f t="shared" ref="H13:H18" si="13">H12+I13</f>
         <v>6.0909999999999513</v>
       </c>
       <c r="I13" s="7">
@@ -2040,7 +2073,7 @@
         <v>1.6879999999999882</v>
       </c>
       <c r="J13" s="7">
-        <f>J12+K13</f>
+        <f t="shared" ref="J13:J18" si="14">J12+K13</f>
         <v>1.089999999999975</v>
       </c>
       <c r="K13" s="7">
@@ -2086,7 +2119,7 @@
         <v>46080</v>
       </c>
       <c r="B14" s="7">
-        <f>B13+C14</f>
+        <f t="shared" si="10"/>
         <v>-8.9009762565925854E-2</v>
       </c>
       <c r="C14" s="7">
@@ -2094,7 +2127,7 @@
         <v>-0.26999999999999957</v>
       </c>
       <c r="D14" s="7">
-        <f>D13+E14</f>
+        <f t="shared" si="11"/>
         <v>-0.31054442339549837</v>
       </c>
       <c r="E14" s="7">
@@ -2102,7 +2135,7 @@
         <v>-8.9999999999999858E-2</v>
       </c>
       <c r="F14" s="7">
-        <f>F13+G14</f>
+        <f t="shared" si="12"/>
         <v>-2.648030495551934E-2</v>
       </c>
       <c r="G14" s="7">
@@ -2110,7 +2143,7 @@
         <v>-9.9999999999997868E-3</v>
       </c>
       <c r="H14" s="7">
-        <f>H13+I14</f>
+        <f t="shared" si="13"/>
         <v>4.3909999999999059</v>
       </c>
       <c r="I14" s="7">
@@ -2118,7 +2151,7 @@
         <v>-1.7000000000000455</v>
       </c>
       <c r="J14" s="7">
-        <f>J13+K14</f>
+        <f t="shared" si="14"/>
         <v>1.3899999999999864</v>
       </c>
       <c r="K14" s="7">
@@ -2164,7 +2197,7 @@
         <v>46082</v>
       </c>
       <c r="B15" s="7">
-        <f>B14+C15</f>
+        <f t="shared" si="10"/>
         <v>0.32099023743407429</v>
       </c>
       <c r="C15" s="7">
@@ -2172,7 +2205,7 @@
         <v>0.41000000000000014</v>
       </c>
       <c r="D15" s="7">
-        <f>D14+E15</f>
+        <f t="shared" si="11"/>
         <v>-0.47054442339549851</v>
       </c>
       <c r="E15" s="7">
@@ -2180,7 +2213,7 @@
         <v>-0.16000000000000014</v>
       </c>
       <c r="F15" s="7">
-        <f>F14+G15</f>
+        <f t="shared" si="12"/>
         <v>-4.6480304955519358E-2</v>
       </c>
       <c r="G15" s="7">
@@ -2188,7 +2221,7 @@
         <v>-2.0000000000000018E-2</v>
       </c>
       <c r="H15" s="7">
-        <f>H14+I15</f>
+        <f t="shared" si="13"/>
         <v>5.2509999999999195</v>
       </c>
       <c r="I15" s="7">
@@ -2196,7 +2229,7 @@
         <v>0.86000000000001364</v>
       </c>
       <c r="J15" s="7">
-        <f>J14+K15</f>
+        <f t="shared" si="14"/>
         <v>1.5400000000000205</v>
       </c>
       <c r="K15" s="7">
@@ -2242,7 +2275,7 @@
         <v>46085</v>
       </c>
       <c r="B16" s="7">
-        <f>B15+C16</f>
+        <f t="shared" si="10"/>
         <v>0.40099023743407258</v>
       </c>
       <c r="C16" s="7">
@@ -2250,7 +2283,7 @@
         <v>7.9999999999998295E-2</v>
       </c>
       <c r="D16" s="7">
-        <f>D15+E16</f>
+        <f t="shared" si="11"/>
         <v>-0.6205444233955042</v>
       </c>
       <c r="E16" s="7">
@@ -2258,7 +2291,7 @@
         <v>-0.15000000000000568</v>
       </c>
       <c r="F16" s="7">
-        <f>F15+G16</f>
+        <f t="shared" si="12"/>
         <v>-7.6480304955519163E-2</v>
       </c>
       <c r="G16" s="7">
@@ -2266,7 +2299,7 @@
         <v>-2.9999999999999805E-2</v>
       </c>
       <c r="H16" s="7">
-        <f>H15+I16</f>
+        <f t="shared" si="13"/>
         <v>5.4209999999999354</v>
       </c>
       <c r="I16" s="7">
@@ -2274,7 +2307,7 @@
         <v>0.17000000000001592</v>
       </c>
       <c r="J16" s="7">
-        <f>J15+K16</f>
+        <f t="shared" si="14"/>
         <v>1.4399999999999977</v>
       </c>
       <c r="K16" s="7">
@@ -2320,7 +2353,7 @@
         <v>46086</v>
       </c>
       <c r="B17" s="7">
-        <f>B16+C17</f>
+        <f t="shared" si="10"/>
         <v>0.4419902374340694</v>
       </c>
       <c r="C17" s="7">
@@ -2328,7 +2361,7 @@
         <v>4.0999999999996817E-2</v>
       </c>
       <c r="D17" s="7">
-        <f>D16+E17</f>
+        <f t="shared" si="11"/>
         <v>-0.68454442339550425</v>
       </c>
       <c r="E17" s="7">
@@ -2336,7 +2369,7 @@
         <v>-6.4000000000000057E-2</v>
       </c>
       <c r="F17" s="7">
-        <f>F16+G17</f>
+        <f t="shared" si="12"/>
         <v>-0.24348030495551898</v>
       </c>
       <c r="G17" s="7">
@@ -2344,7 +2377,7 @@
         <v>-0.16699999999999982</v>
       </c>
       <c r="H17" s="7">
-        <f>H16+I17</f>
+        <f t="shared" si="13"/>
         <v>4.446999999999889</v>
       </c>
       <c r="I17" s="7">
@@ -2352,7 +2385,7 @@
         <v>-0.97400000000004638</v>
       </c>
       <c r="J17" s="7">
-        <f>J16+K17</f>
+        <f t="shared" si="14"/>
         <v>2.9399999999999977</v>
       </c>
       <c r="K17" s="7">
@@ -2398,43 +2431,43 @@
         <v>46087</v>
       </c>
       <c r="B18" s="7">
-        <f>B17+C18</f>
+        <f t="shared" si="10"/>
         <v>0.40899023743406815</v>
       </c>
       <c r="C18" s="7">
-        <f t="shared" ref="C18" si="10">B9-C9</f>
+        <f t="shared" ref="C18" si="15">B9-C9</f>
         <v>-3.3000000000001251E-2</v>
       </c>
       <c r="D18" s="7">
-        <f>D17+E18</f>
+        <f t="shared" si="11"/>
         <v>-0.73054442339550363</v>
       </c>
       <c r="E18" s="7">
-        <f t="shared" ref="E18" si="11">D9-E9</f>
+        <f t="shared" ref="E18" si="16">D9-E9</f>
         <v>-4.5999999999999375E-2</v>
       </c>
       <c r="F18" s="7">
-        <f>F17+G18</f>
+        <f t="shared" si="12"/>
         <v>-0.25648030495551888</v>
       </c>
       <c r="G18" s="7">
-        <f t="shared" ref="G18" si="12">F9-G9</f>
+        <f t="shared" ref="G18" si="17">F9-G9</f>
         <v>-1.2999999999999901E-2</v>
       </c>
       <c r="H18" s="7">
-        <f>H17+I18</f>
+        <f t="shared" si="13"/>
         <v>1.2289999999998713</v>
       </c>
       <c r="I18" s="7">
-        <f t="shared" ref="I18" si="13">H9-I9</f>
+        <f t="shared" ref="I18" si="18">H9-I9</f>
         <v>-3.2180000000000177</v>
       </c>
       <c r="J18" s="7">
-        <f>J17+K18</f>
+        <f t="shared" si="14"/>
         <v>7.0400000000000205</v>
       </c>
       <c r="K18" s="7">
-        <f t="shared" ref="K18" si="14">J9-K9</f>
+        <f t="shared" ref="K18" si="19">J9-K9</f>
         <v>4.1000000000000227</v>
       </c>
       <c r="L18" s="7"/>
@@ -2564,7 +2597,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D45F4E0-DDC0-44AE-A48F-B33A7D849191}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="73.54296875" customWidth="1"/>
@@ -2576,16 +2609,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="23"/>
+      <c r="C1" s="25"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="17" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2603,7 +2636,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
-        <f t="shared" ref="A4:A33" si="0">"UPDATE Productes SET TickerExchange = '"&amp;C4&amp;"' WHERE Id = "&amp;B4&amp;";"</f>
+        <f t="shared" ref="A4:A38" si="0">"UPDATE Productes SET TickerExchange = '"&amp;C4&amp;"' WHERE Id = "&amp;B4&amp;";"</f>
         <v>UPDATE Productes SET TickerExchange = 'LU0231459107.EUFUND' WHERE Id = 3;</v>
       </c>
       <c r="B4" s="16">
@@ -2894,159 +2927,291 @@
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="str">
         <f t="shared" si="0"/>
-        <v>UPDATE Productes SET TickerExchange = 'CLAR.US' WHERE Id = 1045;</v>
-      </c>
-      <c r="B28" s="16">
-        <v>1045</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>43</v>
+        <v>UPDATE Productes SET TickerExchange = 'MTS.AU' WHERE Id = 7;</v>
+      </c>
+      <c r="B28" s="15">
+        <v>7</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
         <f t="shared" si="0"/>
-        <v>UPDATE Productes SET TickerExchange = 'LU1965927921.EUFUND' WHERE Id = 1046;</v>
-      </c>
-      <c r="B29" s="16">
-        <v>1046</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>78</v>
+        <v>UPDATE Productes SET TickerExchange = 'SAN.MC' WHERE Id = 8;</v>
+      </c>
+      <c r="B29" s="15">
+        <v>8</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="str">
         <f t="shared" si="0"/>
-        <v>UPDATE Productes SET TickerExchange = 'M4I.MU' WHERE Id = 1053;</v>
-      </c>
-      <c r="B30" s="16">
-        <v>1053</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>44</v>
+        <v>UPDATE Productes SET TickerExchange = 'TEF.MC' WHERE Id = 9;</v>
+      </c>
+      <c r="B30" s="15">
+        <v>9</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="str">
         <f t="shared" si="0"/>
-        <v>UPDATE Productes SET TickerExchange = 'BRYN.XETRA' WHERE Id = 1054;</v>
-      </c>
-      <c r="B31" s="16">
-        <v>1054</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>45</v>
+        <v>UPDATE Productes SET TickerExchange = 'SAB.VN' WHERE Id = 22;</v>
+      </c>
+      <c r="B31" s="15">
+        <v>22</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="str">
         <f t="shared" si="0"/>
-        <v>UPDATE Productes SET TickerExchange = 'NVO.US' WHERE Id = 1058;</v>
-      </c>
-      <c r="B32" s="16">
-        <v>1058</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>47</v>
+        <v>UPDATE Productes SET TickerExchange = 'ITX.MC' WHERE Id = 23;</v>
+      </c>
+      <c r="B32" s="15">
+        <v>23</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="str">
         <f t="shared" si="0"/>
-        <v>UPDATE Productes SET TickerExchange = 'NOVO-B.CO' WHERE Id = 1059;</v>
+        <v>UPDATE Productes SET TickerExchange = 'CLAR.US' WHERE Id = 1045;</v>
       </c>
       <c r="B33" s="16">
-        <v>1059</v>
+        <v>1045</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
+      <c r="A34" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'LU1965927921.EUFUND' WHERE Id = 1046;</v>
+      </c>
+      <c r="B34" s="16">
+        <v>1046</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B35" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="C35" s="23"/>
+      <c r="A35" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'M4I.MU' WHERE Id = 1053;</v>
+      </c>
+      <c r="B35" s="16">
+        <v>1053</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B36" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C36" s="24" t="s">
-        <v>6</v>
+      <c r="A36" t="str">
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'BRYN.XETRA' WHERE Id = 1054;</v>
+      </c>
+      <c r="B36" s="16">
+        <v>1054</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="str">
-        <f>"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C37&amp;"' WHERE Id = "&amp;B37&amp;";"</f>
-        <v>UPDATE Productes_ProdAccions SET Ticker = 'CLAR' WHERE Id = 1045;</v>
-      </c>
-      <c r="B37" s="15">
-        <v>1045</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>42</v>
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'NVO.US' WHERE Id = 1058;</v>
+      </c>
+      <c r="B37" s="16">
+        <v>1058</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
-        <f t="shared" ref="A38:A41" si="1">"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C38&amp;"' WHERE Id = "&amp;B38&amp;";"</f>
+        <f t="shared" si="0"/>
+        <v>UPDATE Productes SET TickerExchange = 'NOVO-B.CO' WHERE Id = 1059;</v>
+      </c>
+      <c r="B38" s="16">
+        <v>1059</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B40" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="25"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B41" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="str">
+        <f t="shared" ref="A42:A47" si="1">"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C42&amp;"' WHERE Id = "&amp;B42&amp;";"</f>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'MTS' WHERE Id = 7;</v>
+      </c>
+      <c r="B42" s="15">
+        <v>7</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'SAN' WHERE Id = 8;</v>
+      </c>
+      <c r="B43" s="15">
+        <v>8</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'TEF' WHERE Id = 9;</v>
+      </c>
+      <c r="B44" s="15">
+        <v>9</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'SAB' WHERE Id = 22;</v>
+      </c>
+      <c r="B45" s="15">
+        <v>22</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'ITX' WHERE Id = 23;</v>
+      </c>
+      <c r="B46" s="15">
+        <v>23</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" t="str">
+        <f t="shared" si="1"/>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'NDUEEGF' WHERE Id = 24;</v>
+      </c>
+      <c r="B47" s="15">
+        <v>24</v>
+      </c>
+      <c r="C47" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="str">
+        <f>"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C48&amp;"' WHERE Id = "&amp;B48&amp;";"</f>
+        <v>UPDATE Productes_ProdAccions SET Ticker = 'CLAR' WHERE Id = 1045;</v>
+      </c>
+      <c r="B48" s="15">
+        <v>1045</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" t="str">
+        <f t="shared" ref="A49:A52" si="2">"UPDATE Productes_ProdAccions SET Ticker = '"&amp;C49&amp;"' WHERE Id = "&amp;B49&amp;";"</f>
         <v>UPDATE Productes_ProdAccions SET Ticker = 'M4I' WHERE Id = 1053;</v>
       </c>
-      <c r="B38" s="15">
+      <c r="B49" s="15">
         <v>1053</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C49" s="15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" t="str">
-        <f t="shared" si="1"/>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" t="str">
+        <f t="shared" si="2"/>
         <v>UPDATE Productes_ProdAccions SET Ticker = 'BRYN' WHERE Id = 1054;</v>
       </c>
-      <c r="B39" s="15">
+      <c r="B50" s="15">
         <v>1054</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C50" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" t="str">
-        <f t="shared" si="1"/>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" t="str">
+        <f t="shared" si="2"/>
         <v>UPDATE Productes_ProdAccions SET Ticker = 'NVO' WHERE Id = 1058;</v>
       </c>
-      <c r="B40" s="15">
+      <c r="B51" s="15">
         <v>1058</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="C51" s="15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" t="str">
-        <f t="shared" si="1"/>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" t="str">
+        <f t="shared" si="2"/>
         <v>UPDATE Productes_ProdAccions SET Ticker = 'NOVO-B' WHERE Id = 1059;</v>
       </c>
-      <c r="B41" s="15">
+      <c r="B52" s="15">
         <v>1059</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C52" s="15" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B40:C40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Falta canviar el boto esborrar
</commit_message>
<xml_diff>
--- a/Docs/AccesCotitzacionsEodHd.xlsx
+++ b/Docs/AccesCotitzacionsEodHd.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\PC-HP11\naoj61\InversionsV3\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542899D6-0B67-4089-9FB9-3605101340DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B183805-E207-46F1-BF77-B1149AFDF6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12720" activeTab="2" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
+    <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{86B7CC84-E031-4E3A-8474-F905DD073FFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1420,7 +1420,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF80A40C-7CB8-46A0-99EA-6106618D84CF}">
-  <dimension ref="A1:S18"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
@@ -1430,7 +1430,7 @@
     <col min="12" max="19" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
         <v>40</v>
       </c>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="S1" s="20"/>
     </row>
-    <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="24"/>
       <c r="B2" s="5" t="s">
         <v>24</v>
@@ -1528,7 +1528,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="9">
         <v>46078</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>93.21</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A4" s="10">
         <v>46079</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>93.23</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A5" s="10">
         <v>46080</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>93.23</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A6" s="10">
         <v>46082</v>
       </c>
@@ -1753,7 +1753,7 @@
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
         <v>46085</v>
       </c>
@@ -1808,7 +1808,7 @@
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <v>46086</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>93.21</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" s="10">
         <v>46087</v>
       </c>
@@ -1901,343 +1901,275 @@
       <c r="K9" s="18">
         <v>424.95</v>
       </c>
+      <c r="L9" s="18">
+        <v>110.79</v>
+      </c>
       <c r="M9" s="18">
         <v>110.79</v>
       </c>
+      <c r="N9" s="18">
+        <v>475.66340000000002</v>
+      </c>
       <c r="O9" s="18">
         <v>475.66300000000001</v>
       </c>
+      <c r="P9" s="18">
+        <v>56.707900000000002</v>
+      </c>
       <c r="Q9" s="18">
         <v>56.41</v>
       </c>
+      <c r="R9" s="18">
+        <v>93.24</v>
+      </c>
       <c r="S9">
         <v>93.24</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="10"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="7"/>
-      <c r="S10" s="7"/>
-    </row>
-    <row r="11" spans="1:19" ht="24" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="11" t="s">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A10" s="10">
+        <v>46090</v>
+      </c>
+      <c r="B10" s="7">
+        <v>34.049999999999997</v>
+      </c>
+      <c r="C10" s="18">
+        <v>34.07</v>
+      </c>
+      <c r="D10" s="18">
+        <v>34.049999999999997</v>
+      </c>
+      <c r="E10" s="18">
+        <v>34.128</v>
+      </c>
+      <c r="F10" s="18">
+        <v>2.52</v>
+      </c>
+      <c r="G10" s="18">
+        <v>2.5569999999999999</v>
+      </c>
+      <c r="H10" s="18">
+        <v>437.75</v>
+      </c>
+      <c r="I10" s="18">
+        <v>441.86200000000002</v>
+      </c>
+      <c r="J10" s="18">
+        <v>426.9</v>
+      </c>
+      <c r="K10" s="18">
+        <v>425.3</v>
+      </c>
+      <c r="L10" s="18">
+        <v>110.78</v>
+      </c>
+      <c r="M10" s="18">
+        <v>110.78</v>
+      </c>
+      <c r="N10" s="18">
+        <v>475.66300000000001</v>
+      </c>
+      <c r="O10" s="18">
+        <v>475.66300000000001</v>
+      </c>
+      <c r="P10" s="18">
+        <v>56.3566</v>
+      </c>
+      <c r="Q10" s="18">
+        <v>55.868000000000002</v>
+      </c>
+      <c r="R10" s="18">
+        <v>93.22</v>
+      </c>
+      <c r="S10" s="18">
+        <v>93.22</v>
+      </c>
+      <c r="U10" s="18"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11" s="10"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="M11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="Q11" s="18"/>
+    </row>
+    <row r="12" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="10"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="7"/>
+      <c r="R12" s="7"/>
+      <c r="S12" s="7"/>
+    </row>
+    <row r="13" spans="1:21" ht="24" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A13" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="12"/>
-      <c r="S11" s="13"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A12" s="9">
-        <f t="shared" ref="A12:A18" si="0">A3</f>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="13"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A14" s="9">
+        <f t="shared" ref="A14:A21" si="0">A3</f>
         <v>46078</v>
       </c>
-      <c r="B12" s="8">
-        <f>C12</f>
+      <c r="B14" s="8">
+        <f>C14</f>
         <v>0.24695768576897237</v>
       </c>
-      <c r="C12" s="8">
-        <f t="shared" ref="C12:C17" si="1">B3-C3</f>
+      <c r="C14" s="8">
+        <f t="shared" ref="C14:C19" si="1">B3-C3</f>
         <v>0.24695768576897237</v>
       </c>
-      <c r="D12" s="8">
-        <f>E12</f>
+      <c r="D14" s="8">
+        <f>E14</f>
         <v>-0.15269181856709935</v>
       </c>
-      <c r="E12" s="8">
-        <f t="shared" ref="E12:E17" si="2">D3-E3</f>
+      <c r="E14" s="8">
+        <f t="shared" ref="E14:E19" si="2">D3-E3</f>
         <v>-0.15269181856709935</v>
       </c>
-      <c r="F12" s="8">
-        <f>G12</f>
+      <c r="F14" s="8">
+        <f>G14</f>
         <v>-9.9999999999997868E-3</v>
       </c>
-      <c r="G12" s="8">
-        <f t="shared" ref="G12:G17" si="3">F3-G3</f>
+      <c r="G14" s="8">
+        <f t="shared" ref="G14:G19" si="3">F3-G3</f>
         <v>-9.9999999999997868E-3</v>
       </c>
-      <c r="H12" s="8">
-        <f>I12</f>
+      <c r="H14" s="8">
+        <f>I14</f>
         <v>4.4029999999999632</v>
       </c>
-      <c r="I12" s="8">
-        <f t="shared" ref="I12:I17" si="4">H3-I3</f>
+      <c r="I14" s="8">
+        <f t="shared" ref="I14:I19" si="4">H3-I3</f>
         <v>4.4029999999999632</v>
       </c>
-      <c r="J12" s="8">
-        <f>K12</f>
+      <c r="J14" s="8">
+        <f>K14</f>
         <v>0.44999999999998863</v>
       </c>
-      <c r="K12" s="8">
-        <f t="shared" ref="K12:K17" si="5">J3-K3</f>
+      <c r="K14" s="8">
+        <f t="shared" ref="K14:K19" si="5">J3-K3</f>
         <v>0.44999999999998863</v>
       </c>
-      <c r="L12" s="8">
-        <f>M12</f>
+      <c r="L14" s="8">
+        <f>M14</f>
         <v>0</v>
       </c>
-      <c r="M12" s="8">
-        <f t="shared" ref="M12:M17" si="6">L3-M3</f>
+      <c r="M14" s="8">
+        <f t="shared" ref="M14:M21" si="6">L3-M3</f>
         <v>0</v>
       </c>
-      <c r="N12" s="8">
-        <f>O12</f>
+      <c r="N14" s="8">
+        <f>O14</f>
         <v>0</v>
       </c>
-      <c r="O12" s="8">
-        <f t="shared" ref="O12:O17" si="7">N3-O3</f>
+      <c r="O14" s="8">
+        <f t="shared" ref="O14:O21" si="7">N3-O3</f>
         <v>0</v>
       </c>
-      <c r="P12" s="8">
-        <f>Q12</f>
+      <c r="P14" s="8">
+        <f>Q14</f>
         <v>5.2410428147595667E-2</v>
       </c>
-      <c r="Q12" s="8">
-        <f t="shared" ref="Q12:Q17" si="8">P3-Q3</f>
+      <c r="Q14" s="8">
+        <f t="shared" ref="Q14:Q21" si="8">P3-Q3</f>
         <v>5.2410428147595667E-2</v>
       </c>
-      <c r="R12" s="8">
-        <f>S12</f>
+      <c r="R14" s="8">
+        <f>S14</f>
         <v>0</v>
       </c>
-      <c r="S12" s="8">
-        <f t="shared" ref="S12:S17" si="9">R3-S3</f>
+      <c r="S14" s="8">
+        <f t="shared" ref="S14:S21" si="9">R3-S3</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A13" s="10">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A15" s="10">
         <f t="shared" si="0"/>
         <v>46079</v>
       </c>
-      <c r="B13" s="7">
-        <f t="shared" ref="B13:B18" si="10">B12+C13</f>
+      <c r="B15" s="7">
+        <f t="shared" ref="B15:B20" si="10">B14+C15</f>
         <v>0.18099023743407372</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C15" s="7">
         <f t="shared" si="1"/>
         <v>-6.5967448334898648E-2</v>
       </c>
-      <c r="D13" s="7">
-        <f t="shared" ref="D13:D18" si="11">D12+E13</f>
+      <c r="D15" s="7">
+        <f t="shared" ref="D15:D20" si="11">D14+E15</f>
         <v>-0.22054442339549851</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E15" s="7">
         <f t="shared" si="2"/>
         <v>-6.7852604828399166E-2</v>
       </c>
-      <c r="F13" s="7">
-        <f t="shared" ref="F13:F18" si="12">F12+G13</f>
+      <c r="F15" s="7">
+        <f t="shared" ref="F15:F20" si="12">F14+G15</f>
         <v>-1.6480304955519554E-2</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G15" s="7">
         <f t="shared" si="3"/>
         <v>-6.4803049555197667E-3</v>
       </c>
-      <c r="H13" s="7">
-        <f t="shared" ref="H13:H18" si="13">H12+I13</f>
+      <c r="H15" s="7">
+        <f t="shared" ref="H15:H20" si="13">H14+I15</f>
         <v>6.0909999999999513</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I15" s="7">
         <f t="shared" si="4"/>
         <v>1.6879999999999882</v>
       </c>
-      <c r="J13" s="7">
-        <f t="shared" ref="J13:J18" si="14">J12+K13</f>
+      <c r="J15" s="7">
+        <f t="shared" ref="J15:J20" si="14">J14+K15</f>
         <v>1.089999999999975</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K15" s="7">
         <f t="shared" si="5"/>
         <v>0.63999999999998636</v>
       </c>
-      <c r="L13" s="7">
-        <f>L12+M13</f>
-        <v>0</v>
-      </c>
-      <c r="M13" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N13" s="7">
-        <f>N12+O13</f>
-        <v>0</v>
-      </c>
-      <c r="O13" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="P13" s="7">
-        <f>P12+Q13</f>
-        <v>9.7193226838996338E-3</v>
-      </c>
-      <c r="Q13" s="7">
-        <f t="shared" si="8"/>
-        <v>-4.2691105463696033E-2</v>
-      </c>
-      <c r="R13" s="7">
-        <f>R12+S13</f>
-        <v>0</v>
-      </c>
-      <c r="S13" s="7">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A14" s="10">
-        <f t="shared" si="0"/>
-        <v>46080</v>
-      </c>
-      <c r="B14" s="7">
-        <f t="shared" si="10"/>
-        <v>-8.9009762565925854E-2</v>
-      </c>
-      <c r="C14" s="7">
-        <f t="shared" si="1"/>
-        <v>-0.26999999999999957</v>
-      </c>
-      <c r="D14" s="7">
-        <f t="shared" si="11"/>
-        <v>-0.31054442339549837</v>
-      </c>
-      <c r="E14" s="7">
-        <f t="shared" si="2"/>
-        <v>-8.9999999999999858E-2</v>
-      </c>
-      <c r="F14" s="7">
-        <f t="shared" si="12"/>
-        <v>-2.648030495551934E-2</v>
-      </c>
-      <c r="G14" s="7">
-        <f t="shared" si="3"/>
-        <v>-9.9999999999997868E-3</v>
-      </c>
-      <c r="H14" s="7">
-        <f t="shared" si="13"/>
-        <v>4.3909999999999059</v>
-      </c>
-      <c r="I14" s="7">
-        <f t="shared" si="4"/>
-        <v>-1.7000000000000455</v>
-      </c>
-      <c r="J14" s="7">
-        <f t="shared" si="14"/>
-        <v>1.3899999999999864</v>
-      </c>
-      <c r="K14" s="7">
-        <f t="shared" si="5"/>
-        <v>0.30000000000001137</v>
-      </c>
-      <c r="L14" s="7">
-        <f>L13+M14</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="N14" s="7">
-        <f>N13+O14</f>
-        <v>-3.4999999999740794E-3</v>
-      </c>
-      <c r="O14" s="7">
-        <f t="shared" si="7"/>
-        <v>-3.4999999999740794E-3</v>
-      </c>
-      <c r="P14" s="7">
-        <f>P13+Q14</f>
-        <v>6.3919322683901214E-2</v>
-      </c>
-      <c r="Q14" s="7">
-        <f t="shared" si="8"/>
-        <v>5.420000000000158E-2</v>
-      </c>
-      <c r="R14" s="7">
-        <f>R13+S14</f>
-        <v>0</v>
-      </c>
-      <c r="S14" s="7">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A15" s="10">
-        <f t="shared" si="0"/>
-        <v>46082</v>
-      </c>
-      <c r="B15" s="7">
-        <f t="shared" si="10"/>
-        <v>0.32099023743407429</v>
-      </c>
-      <c r="C15" s="7">
-        <f t="shared" si="1"/>
-        <v>0.41000000000000014</v>
-      </c>
-      <c r="D15" s="7">
-        <f t="shared" si="11"/>
-        <v>-0.47054442339549851</v>
-      </c>
-      <c r="E15" s="7">
-        <f t="shared" si="2"/>
-        <v>-0.16000000000000014</v>
-      </c>
-      <c r="F15" s="7">
-        <f t="shared" si="12"/>
-        <v>-4.6480304955519358E-2</v>
-      </c>
-      <c r="G15" s="7">
-        <f t="shared" si="3"/>
-        <v>-2.0000000000000018E-2</v>
-      </c>
-      <c r="H15" s="7">
-        <f t="shared" si="13"/>
-        <v>5.2509999999999195</v>
-      </c>
-      <c r="I15" s="7">
-        <f t="shared" si="4"/>
-        <v>0.86000000000001364</v>
-      </c>
-      <c r="J15" s="7">
-        <f t="shared" si="14"/>
-        <v>1.5400000000000205</v>
-      </c>
-      <c r="K15" s="7">
-        <f t="shared" si="5"/>
-        <v>0.15000000000003411</v>
-      </c>
       <c r="L15" s="7">
-        <f>L14+M15</f>
+        <f t="shared" ref="L15:L20" si="15">L14+M15</f>
         <v>0</v>
       </c>
       <c r="M15" s="7">
@@ -2245,23 +2177,23 @@
         <v>0</v>
       </c>
       <c r="N15" s="7">
-        <f>N14+O15</f>
-        <v>-3.4999999999740794E-3</v>
+        <f t="shared" ref="N15:N20" si="16">N14+O15</f>
+        <v>0</v>
       </c>
       <c r="O15" s="7">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="P15" s="7">
-        <f>P14+Q15</f>
-        <v>6.3919322683901214E-2</v>
+        <f t="shared" ref="P15:P20" si="17">P14+Q15</f>
+        <v>9.7193226838996338E-3</v>
       </c>
       <c r="Q15" s="7">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-4.2691105463696033E-2</v>
       </c>
       <c r="R15" s="7">
-        <f>R14+S15</f>
+        <f t="shared" ref="R15:R20" si="18">R14+S15</f>
         <v>0</v>
       </c>
       <c r="S15" s="7">
@@ -2269,77 +2201,77 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
         <f t="shared" si="0"/>
-        <v>46085</v>
+        <v>46080</v>
       </c>
       <c r="B16" s="7">
         <f t="shared" si="10"/>
-        <v>0.40099023743407258</v>
+        <v>-8.9009762565925854E-2</v>
       </c>
       <c r="C16" s="7">
         <f t="shared" si="1"/>
-        <v>7.9999999999998295E-2</v>
+        <v>-0.26999999999999957</v>
       </c>
       <c r="D16" s="7">
         <f t="shared" si="11"/>
-        <v>-0.6205444233955042</v>
+        <v>-0.31054442339549837</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="2"/>
-        <v>-0.15000000000000568</v>
+        <v>-8.9999999999999858E-2</v>
       </c>
       <c r="F16" s="7">
         <f t="shared" si="12"/>
-        <v>-7.6480304955519163E-2</v>
+        <v>-2.648030495551934E-2</v>
       </c>
       <c r="G16" s="7">
         <f t="shared" si="3"/>
-        <v>-2.9999999999999805E-2</v>
+        <v>-9.9999999999997868E-3</v>
       </c>
       <c r="H16" s="7">
         <f t="shared" si="13"/>
-        <v>5.4209999999999354</v>
+        <v>4.3909999999999059</v>
       </c>
       <c r="I16" s="7">
         <f t="shared" si="4"/>
-        <v>0.17000000000001592</v>
+        <v>-1.7000000000000455</v>
       </c>
       <c r="J16" s="7">
         <f t="shared" si="14"/>
-        <v>1.4399999999999977</v>
+        <v>1.3899999999999864</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="5"/>
-        <v>-0.10000000000002274</v>
+        <v>0.30000000000001137</v>
       </c>
       <c r="L16" s="7">
-        <f>L15+M16</f>
-        <v>1.0000000000005116E-2</v>
+        <f t="shared" si="15"/>
+        <v>0</v>
       </c>
       <c r="M16" s="7">
         <f t="shared" si="6"/>
-        <v>1.0000000000005116E-2</v>
+        <v>0</v>
       </c>
       <c r="N16" s="7">
-        <f>N15+O16</f>
+        <f t="shared" si="16"/>
         <v>-3.4999999999740794E-3</v>
       </c>
       <c r="O16" s="7">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>-3.4999999999740794E-3</v>
       </c>
       <c r="P16" s="7">
-        <f>P15+Q16</f>
-        <v>-0.1848442572435971</v>
+        <f t="shared" si="17"/>
+        <v>6.3919322683901214E-2</v>
       </c>
       <c r="Q16" s="7">
         <f t="shared" si="8"/>
-        <v>-0.24876357992749831</v>
+        <v>5.420000000000158E-2</v>
       </c>
       <c r="R16" s="7">
-        <f>R15+S16</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="S16" s="7">
@@ -2350,130 +2282,392 @@
     <row r="17" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
         <f t="shared" si="0"/>
-        <v>46086</v>
+        <v>46082</v>
       </c>
       <c r="B17" s="7">
         <f t="shared" si="10"/>
-        <v>0.4419902374340694</v>
+        <v>0.32099023743407429</v>
       </c>
       <c r="C17" s="7">
         <f t="shared" si="1"/>
-        <v>4.0999999999996817E-2</v>
+        <v>0.41000000000000014</v>
       </c>
       <c r="D17" s="7">
         <f t="shared" si="11"/>
-        <v>-0.68454442339550425</v>
+        <v>-0.47054442339549851</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="2"/>
-        <v>-6.4000000000000057E-2</v>
+        <v>-0.16000000000000014</v>
       </c>
       <c r="F17" s="7">
         <f t="shared" si="12"/>
-        <v>-0.24348030495551898</v>
+        <v>-4.6480304955519358E-2</v>
       </c>
       <c r="G17" s="7">
         <f t="shared" si="3"/>
-        <v>-0.16699999999999982</v>
+        <v>-2.0000000000000018E-2</v>
       </c>
       <c r="H17" s="7">
         <f t="shared" si="13"/>
-        <v>4.446999999999889</v>
+        <v>5.2509999999999195</v>
       </c>
       <c r="I17" s="7">
         <f t="shared" si="4"/>
-        <v>-0.97400000000004638</v>
+        <v>0.86000000000001364</v>
       </c>
       <c r="J17" s="7">
         <f t="shared" si="14"/>
-        <v>2.9399999999999977</v>
+        <v>1.5400000000000205</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="5"/>
-        <v>1.5</v>
+        <v>0.15000000000003411</v>
       </c>
       <c r="L17" s="7">
-        <f>L16+M17</f>
-        <v>1.0000000000005116E-2</v>
+        <f t="shared" si="15"/>
+        <v>0</v>
       </c>
       <c r="M17" s="7">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N17" s="7">
-        <f>N16+O17</f>
-        <v>-3.999999999962256E-3</v>
+        <f t="shared" si="16"/>
+        <v>-3.4999999999740794E-3</v>
       </c>
       <c r="O17" s="7">
         <f t="shared" si="7"/>
-        <v>-4.9999999998817657E-4</v>
+        <v>0</v>
       </c>
       <c r="P17" s="7">
-        <f>P16+Q17</f>
-        <v>-0.13504425724359947</v>
+        <f t="shared" si="17"/>
+        <v>6.3919322683901214E-2</v>
       </c>
       <c r="Q17" s="7">
         <f t="shared" si="8"/>
-        <v>4.9799999999997624E-2</v>
+        <v>0</v>
       </c>
       <c r="R17" s="7">
-        <f>R16+S17</f>
-        <v>3.0000000000001137E-2</v>
+        <f t="shared" si="18"/>
+        <v>0</v>
       </c>
       <c r="S17" s="7">
         <f t="shared" si="9"/>
-        <v>3.0000000000001137E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
         <f t="shared" si="0"/>
-        <v>46087</v>
+        <v>46085</v>
       </c>
       <c r="B18" s="7">
         <f t="shared" si="10"/>
-        <v>0.40899023743406815</v>
+        <v>0.40099023743407258</v>
       </c>
       <c r="C18" s="7">
-        <f t="shared" ref="C18" si="15">B9-C9</f>
-        <v>-3.3000000000001251E-2</v>
+        <f t="shared" si="1"/>
+        <v>7.9999999999998295E-2</v>
       </c>
       <c r="D18" s="7">
         <f t="shared" si="11"/>
-        <v>-0.73054442339550363</v>
+        <v>-0.6205444233955042</v>
       </c>
       <c r="E18" s="7">
-        <f t="shared" ref="E18" si="16">D9-E9</f>
-        <v>-4.5999999999999375E-2</v>
+        <f t="shared" si="2"/>
+        <v>-0.15000000000000568</v>
       </c>
       <c r="F18" s="7">
         <f t="shared" si="12"/>
-        <v>-0.25648030495551888</v>
+        <v>-7.6480304955519163E-2</v>
       </c>
       <c r="G18" s="7">
-        <f t="shared" ref="G18" si="17">F9-G9</f>
-        <v>-1.2999999999999901E-2</v>
+        <f t="shared" si="3"/>
+        <v>-2.9999999999999805E-2</v>
       </c>
       <c r="H18" s="7">
         <f t="shared" si="13"/>
-        <v>1.2289999999998713</v>
+        <v>5.4209999999999354</v>
       </c>
       <c r="I18" s="7">
-        <f t="shared" ref="I18" si="18">H9-I9</f>
-        <v>-3.2180000000000177</v>
+        <f t="shared" si="4"/>
+        <v>0.17000000000001592</v>
       </c>
       <c r="J18" s="7">
         <f t="shared" si="14"/>
+        <v>1.4399999999999977</v>
+      </c>
+      <c r="K18" s="7">
+        <f t="shared" si="5"/>
+        <v>-0.10000000000002274</v>
+      </c>
+      <c r="L18" s="7">
+        <f t="shared" si="15"/>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="M18" s="7">
+        <f t="shared" si="6"/>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="N18" s="7">
+        <f t="shared" si="16"/>
+        <v>-3.4999999999740794E-3</v>
+      </c>
+      <c r="O18" s="7">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="P18" s="7">
+        <f t="shared" si="17"/>
+        <v>-0.1848442572435971</v>
+      </c>
+      <c r="Q18" s="7">
+        <f t="shared" si="8"/>
+        <v>-0.24876357992749831</v>
+      </c>
+      <c r="R18" s="7">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="S18" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A19" s="10">
+        <f t="shared" si="0"/>
+        <v>46086</v>
+      </c>
+      <c r="B19" s="7">
+        <f t="shared" si="10"/>
+        <v>0.4419902374340694</v>
+      </c>
+      <c r="C19" s="7">
+        <f t="shared" si="1"/>
+        <v>4.0999999999996817E-2</v>
+      </c>
+      <c r="D19" s="7">
+        <f t="shared" si="11"/>
+        <v>-0.68454442339550425</v>
+      </c>
+      <c r="E19" s="7">
+        <f t="shared" si="2"/>
+        <v>-6.4000000000000057E-2</v>
+      </c>
+      <c r="F19" s="7">
+        <f t="shared" si="12"/>
+        <v>-0.24348030495551898</v>
+      </c>
+      <c r="G19" s="7">
+        <f t="shared" si="3"/>
+        <v>-0.16699999999999982</v>
+      </c>
+      <c r="H19" s="7">
+        <f t="shared" si="13"/>
+        <v>4.446999999999889</v>
+      </c>
+      <c r="I19" s="7">
+        <f t="shared" si="4"/>
+        <v>-0.97400000000004638</v>
+      </c>
+      <c r="J19" s="7">
+        <f t="shared" si="14"/>
+        <v>2.9399999999999977</v>
+      </c>
+      <c r="K19" s="7">
+        <f t="shared" si="5"/>
+        <v>1.5</v>
+      </c>
+      <c r="L19" s="7">
+        <f t="shared" si="15"/>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="M19" s="7">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N19" s="7">
+        <f t="shared" si="16"/>
+        <v>-3.999999999962256E-3</v>
+      </c>
+      <c r="O19" s="7">
+        <f t="shared" si="7"/>
+        <v>-4.9999999998817657E-4</v>
+      </c>
+      <c r="P19" s="7">
+        <f t="shared" si="17"/>
+        <v>-0.13504425724359947</v>
+      </c>
+      <c r="Q19" s="7">
+        <f t="shared" si="8"/>
+        <v>4.9799999999997624E-2</v>
+      </c>
+      <c r="R19" s="7">
+        <f t="shared" si="18"/>
+        <v>3.0000000000001137E-2</v>
+      </c>
+      <c r="S19" s="7">
+        <f t="shared" si="9"/>
+        <v>3.0000000000001137E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A20" s="10">
+        <f t="shared" si="0"/>
+        <v>46087</v>
+      </c>
+      <c r="B20" s="7">
+        <f t="shared" si="10"/>
+        <v>0.40899023743406815</v>
+      </c>
+      <c r="C20" s="7">
+        <f t="shared" ref="C20" si="19">B9-C9</f>
+        <v>-3.3000000000001251E-2</v>
+      </c>
+      <c r="D20" s="7">
+        <f t="shared" si="11"/>
+        <v>-0.73054442339550363</v>
+      </c>
+      <c r="E20" s="7">
+        <f t="shared" ref="E20" si="20">D9-E9</f>
+        <v>-4.5999999999999375E-2</v>
+      </c>
+      <c r="F20" s="7">
+        <f t="shared" si="12"/>
+        <v>-0.25648030495551888</v>
+      </c>
+      <c r="G20" s="7">
+        <f t="shared" ref="G20" si="21">F9-G9</f>
+        <v>-1.2999999999999901E-2</v>
+      </c>
+      <c r="H20" s="7">
+        <f t="shared" si="13"/>
+        <v>1.2289999999998713</v>
+      </c>
+      <c r="I20" s="7">
+        <f t="shared" ref="I20" si="22">H9-I9</f>
+        <v>-3.2180000000000177</v>
+      </c>
+      <c r="J20" s="7">
+        <f t="shared" si="14"/>
         <v>7.0400000000000205</v>
       </c>
-      <c r="K18" s="7">
-        <f t="shared" ref="K18" si="19">J9-K9</f>
+      <c r="K20" s="7">
+        <f t="shared" ref="K20" si="23">J9-K9</f>
         <v>4.1000000000000227</v>
       </c>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
+      <c r="L20" s="7">
+        <f t="shared" si="15"/>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="M20" s="7">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N20" s="7">
+        <f t="shared" si="16"/>
+        <v>-3.5999999999489773E-3</v>
+      </c>
+      <c r="O20" s="7">
+        <f t="shared" si="7"/>
+        <v>4.0000000001327862E-4</v>
+      </c>
+      <c r="P20" s="7">
+        <f t="shared" si="17"/>
+        <v>0.16285574275640613</v>
+      </c>
+      <c r="Q20" s="7">
+        <f t="shared" si="8"/>
+        <v>0.2979000000000056</v>
+      </c>
+      <c r="R20" s="7">
+        <f t="shared" si="18"/>
+        <v>3.0000000000001137E-2</v>
+      </c>
+      <c r="S20" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A21" s="10">
+        <f t="shared" si="0"/>
+        <v>46090</v>
+      </c>
+      <c r="B21" s="7">
+        <f t="shared" ref="B21" si="24">B20+C21</f>
+        <v>0.38899023743406502</v>
+      </c>
+      <c r="C21" s="7">
+        <f t="shared" ref="C21" si="25">B10-C10</f>
+        <v>-2.0000000000003126E-2</v>
+      </c>
+      <c r="D21" s="7">
+        <f t="shared" ref="D21" si="26">D20+E21</f>
+        <v>-0.80854442339550658</v>
+      </c>
+      <c r="E21" s="7">
+        <f t="shared" ref="E21" si="27">D10-E10</f>
+        <v>-7.8000000000002956E-2</v>
+      </c>
+      <c r="F21" s="7">
+        <f t="shared" ref="F21" si="28">F20+G21</f>
+        <v>-0.2934803049555188</v>
+      </c>
+      <c r="G21" s="7">
+        <f t="shared" ref="G21" si="29">F10-G10</f>
+        <v>-3.6999999999999922E-2</v>
+      </c>
+      <c r="H21" s="7">
+        <f t="shared" ref="H21" si="30">H20+I21</f>
+        <v>-2.8830000000001519</v>
+      </c>
+      <c r="I21" s="7">
+        <f t="shared" ref="I21" si="31">H10-I10</f>
+        <v>-4.1120000000000232</v>
+      </c>
+      <c r="J21" s="7">
+        <f t="shared" ref="J21" si="32">J20+K21</f>
+        <v>8.6399999999999864</v>
+      </c>
+      <c r="K21" s="7">
+        <f t="shared" ref="K21" si="33">J10-K10</f>
+        <v>1.5999999999999659</v>
+      </c>
+      <c r="L21" s="7">
+        <f t="shared" ref="L21" si="34">L20+M21</f>
+        <v>1.0000000000005116E-2</v>
+      </c>
+      <c r="M21" s="7">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N21" s="7">
+        <f t="shared" ref="N21" si="35">N20+O21</f>
+        <v>-3.5999999999489773E-3</v>
+      </c>
+      <c r="O21" s="7">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="P21" s="7">
+        <f t="shared" ref="P21" si="36">P20+Q21</f>
+        <v>0.65145574275640428</v>
+      </c>
+      <c r="Q21" s="7">
+        <f t="shared" si="8"/>
+        <v>0.48859999999999815</v>
+      </c>
+      <c r="R21" s="7">
+        <f t="shared" ref="R21" si="37">R20+S21</f>
+        <v>3.0000000000001137E-2</v>
+      </c>
+      <c r="S21" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2488,109 +2682,109 @@
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C12:C18">
+  <conditionalFormatting sqref="C14:C21">
     <cfRule type="expression" dxfId="26" priority="25">
-      <formula>AND(C12&gt;-1, C12&lt; 1, C12 &lt;&gt; 0)</formula>
+      <formula>AND(C14&gt;-1, C14&lt; 1, C14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="25" priority="26">
-      <formula>C12&lt;=-1</formula>
+      <formula>C14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="24" priority="27">
-      <formula>C12&gt;=1</formula>
+      <formula>C14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E12:E18">
+  <conditionalFormatting sqref="E14:E21">
     <cfRule type="expression" dxfId="23" priority="28">
-      <formula>AND(E12&gt;-1, E12&lt; 1, E12 &lt;&gt; 0)</formula>
+      <formula>AND(E14&gt;-1, E14&lt; 1, E14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="22" priority="29">
-      <formula>E12&lt;=-1</formula>
+      <formula>E14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="21" priority="30">
-      <formula>E12&gt;=1</formula>
+      <formula>E14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G12:G18">
+  <conditionalFormatting sqref="G14:G21">
     <cfRule type="expression" dxfId="20" priority="22">
-      <formula>AND(G12&gt;-1, G12&lt; 1, G12 &lt;&gt; 0)</formula>
+      <formula>AND(G14&gt;-1, G14&lt; 1, G14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="19" priority="23">
-      <formula>G12&lt;=-1</formula>
+      <formula>G14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="18" priority="24">
-      <formula>G12&gt;=1</formula>
+      <formula>G14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I12:I18">
+  <conditionalFormatting sqref="I14:I21">
     <cfRule type="expression" dxfId="17" priority="19">
-      <formula>AND(I12&gt;-1, I12&lt; 1, I12 &lt;&gt; 0)</formula>
+      <formula>AND(I14&gt;-1, I14&lt; 1, I14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="16" priority="20">
-      <formula>I12&lt;=-1</formula>
+      <formula>I14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="15" priority="21">
-      <formula>I12&gt;=1</formula>
+      <formula>I14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K12:K18">
+  <conditionalFormatting sqref="K14:K21">
     <cfRule type="expression" dxfId="14" priority="16">
-      <formula>AND(K12&gt;-1, K12&lt; 1, K12 &lt;&gt; 0)</formula>
+      <formula>AND(K14&gt;-1, K14&lt; 1, K14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="13" priority="17">
-      <formula>K12&lt;=-1</formula>
+      <formula>K14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="12" priority="18">
-      <formula>K12&gt;=1</formula>
+      <formula>K14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M12:M18">
+  <conditionalFormatting sqref="M14:M21">
     <cfRule type="expression" dxfId="11" priority="10">
-      <formula>AND(M12&gt;-1, M12&lt; 1, M12 &lt;&gt; 0)</formula>
+      <formula>AND(M14&gt;-1, M14&lt; 1, M14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="10" priority="11">
-      <formula>M12&lt;=-1</formula>
+      <formula>M14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="9" priority="12">
-      <formula>M12&gt;=1</formula>
+      <formula>M14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O12:O18">
+  <conditionalFormatting sqref="O14:O21">
     <cfRule type="expression" dxfId="8" priority="7">
-      <formula>AND(O12&gt;-1, O12&lt; 1, O12 &lt;&gt; 0)</formula>
+      <formula>AND(O14&gt;-1, O14&lt; 1, O14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="7" priority="8">
-      <formula>O12&lt;=-1</formula>
+      <formula>O14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="6" priority="9">
-      <formula>O12&gt;=1</formula>
+      <formula>O14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q12:Q17">
+  <conditionalFormatting sqref="Q14:Q21">
     <cfRule type="expression" dxfId="5" priority="4">
-      <formula>AND(Q12&gt;-1, Q12&lt; 1, Q12 &lt;&gt; 0)</formula>
+      <formula>AND(Q14&gt;-1, Q14&lt; 1, Q14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="4" priority="5">
-      <formula>Q12&lt;=-1</formula>
+      <formula>Q14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="3" priority="6">
-      <formula>Q12&gt;=1</formula>
+      <formula>Q14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S12:S17">
+  <conditionalFormatting sqref="S14:S21">
     <cfRule type="expression" dxfId="2" priority="1">
-      <formula>AND(S12&gt;-1, S12&lt; 1, S12 &lt;&gt; 0)</formula>
+      <formula>AND(S14&gt;-1, S14&lt; 1, S14 &lt;&gt; 0)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>S12&lt;=-1</formula>
+      <formula>S14&lt;=-1</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="3">
-      <formula>S12&gt;=1</formula>
+      <formula>S14&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="F12:K14 L12:R14 E12:E16 G15:Q16 F15:F16 R15:T16" formula="1"/>
+    <ignoredError sqref="F14:K16 L14:R16 E14:E18 G17:Q18 F17:F18 R17:T18" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>